<commit_message>
Add 'Development FD Spread' sheet: individual vs institutional FD by tenure
</commit_message>
<xml_diff>
--- a/reports/Interest_Rate_Summary.xlsx
+++ b/reports/Interest_Rate_Summary.xlsx
@@ -8,12 +8,14 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interest Rate Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly History" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development FD Spread" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly History" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Interest Rate Summary'!$A$4:$AB$39</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Monthly History'!$A$1:$N$67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Development FD Spread'!$A$4:$V$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Monthly History'!$A$1:$N$67</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -114,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -159,6 +161,8 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -4213,6 +4217,1291 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:V19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Development Banks — Fixed Deposit: Individual vs Institutional (Ashwin 2083)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>3 Months</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>6 Months</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>1 Year (12 Months)</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="n"/>
+      <c r="J3" s="2" t="n"/>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>2 Years</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="n"/>
+      <c r="M3" s="2" t="n"/>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>3 Years</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="n"/>
+      <c r="P3" s="2" t="n"/>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>4 Years</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="n"/>
+      <c r="S3" s="2" t="n"/>
+      <c r="T3" s="2" t="inlineStr">
+        <is>
+          <t>5 Years &amp; Above</t>
+        </is>
+      </c>
+      <c r="U3" s="2" t="n"/>
+      <c r="V3" s="2" t="n"/>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="3" t="n"/>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Individual</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Institutional</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Difference</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Individual</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Institutional</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Difference</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Individual</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Institutional</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Difference</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>Individual</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Institutional</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>Difference</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>Individual</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>Institutional</t>
+        </is>
+      </c>
+      <c r="P4" s="4" t="inlineStr">
+        <is>
+          <t>Difference</t>
+        </is>
+      </c>
+      <c r="Q4" s="3" t="inlineStr">
+        <is>
+          <t>Individual</t>
+        </is>
+      </c>
+      <c r="R4" s="3" t="inlineStr">
+        <is>
+          <t>Institutional</t>
+        </is>
+      </c>
+      <c r="S4" s="4" t="inlineStr">
+        <is>
+          <t>Difference</t>
+        </is>
+      </c>
+      <c r="T4" s="3" t="inlineStr">
+        <is>
+          <t>Individual</t>
+        </is>
+      </c>
+      <c r="U4" s="3" t="inlineStr">
+        <is>
+          <t>Institutional</t>
+        </is>
+      </c>
+      <c r="V4" s="4" t="inlineStr">
+        <is>
+          <t>Difference</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>Corporate Development Bank Ltd.</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="D5" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>0.0375</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>0.0285</v>
+      </c>
+      <c r="G5" s="9" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="H5" s="8" t="n">
+        <v>0.0425</v>
+      </c>
+      <c r="I5" s="8" t="n">
+        <v>0.0325</v>
+      </c>
+      <c r="J5" s="9" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="K5" s="8" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="L5" s="8" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="M5" s="9" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="N5" s="8" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="O5" s="8" t="n">
+        <v>0.0425</v>
+      </c>
+      <c r="P5" s="9" t="n">
+        <v>0.0075</v>
+      </c>
+      <c r="Q5" s="8" t="n">
+        <v>0.0525</v>
+      </c>
+      <c r="R5" s="8" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="S5" s="9" t="n">
+        <v>0.0075</v>
+      </c>
+      <c r="T5" s="8" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="U5" s="8" t="n">
+        <v>0.0475</v>
+      </c>
+      <c r="V5" s="9" t="n">
+        <v>0.0075</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>Garima Bikas Bank Ltd.</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="F6" s="12" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="G6" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="12" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="I6" s="12" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="J6" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="12" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="L6" s="12" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="M6" s="13" t="n">
+        <v>0.0025</v>
+      </c>
+      <c r="N6" s="12" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="O6" s="12" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="P6" s="13" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="Q6" s="12" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="R6" s="12" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="S6" s="13" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="T6" s="12" t="n">
+        <v>0.0428</v>
+      </c>
+      <c r="U6" s="12" t="n">
+        <v>0.0325</v>
+      </c>
+      <c r="V6" s="13" t="n">
+        <v>0.0103</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>Green Development Bank Ltd.</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="D7" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="F7" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="G7" s="9" t="n">
+        <v>0.0075</v>
+      </c>
+      <c r="H7" s="8" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="I7" s="8" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="J7" s="9" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="K7" s="8" t="n">
+        <v>0.0475</v>
+      </c>
+      <c r="L7" s="8" t="n">
+        <v>0.0375</v>
+      </c>
+      <c r="M7" s="9" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="N7" s="8" t="n">
+        <v>0.0475</v>
+      </c>
+      <c r="O7" s="8" t="n">
+        <v>0.0375</v>
+      </c>
+      <c r="P7" s="9" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="Q7" s="8" t="n">
+        <v>0.0525</v>
+      </c>
+      <c r="R7" s="8" t="n">
+        <v>0.0425</v>
+      </c>
+      <c r="S7" s="9" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="T7" s="8" t="n">
+        <v>0.0525</v>
+      </c>
+      <c r="U7" s="8" t="n">
+        <v>0.0425</v>
+      </c>
+      <c r="V7" s="9" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t>Jyoti Bikas Bank Ltd.</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="F8" s="12" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="G8" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="12" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="I8" s="12" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="J8" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="12" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="L8" s="12" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="M8" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="12" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="O8" s="12" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="P8" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="12" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="R8" s="12" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="S8" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" s="12" t="n">
+        <v>0.0428</v>
+      </c>
+      <c r="U8" s="12" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="V8" s="13" t="n">
+        <v>0.0153</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>Kamana Sewa Bikas Bank Ltd.</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="C9" s="15" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="D9" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="F9" s="15" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="G9" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="I9" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="J9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="8" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="L9" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="M9" s="9" t="n">
+        <v>0.0025</v>
+      </c>
+      <c r="N9" s="8" t="n">
+        <v>0.0315</v>
+      </c>
+      <c r="O9" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="P9" s="9" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="Q9" s="8" t="n">
+        <v>0.0315</v>
+      </c>
+      <c r="R9" s="8" t="n">
+        <v>0.0335</v>
+      </c>
+      <c r="S9" s="9" t="n">
+        <v>-0.002</v>
+      </c>
+      <c r="T9" s="8" t="n">
+        <v>0.0428</v>
+      </c>
+      <c r="U9" s="8" t="n">
+        <v>0.0335</v>
+      </c>
+      <c r="V9" s="9" t="n">
+        <v>0.009299999999999999</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>Lumbini Bikas Bank Ltd.</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="n">
+        <v>0.028</v>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="n">
+        <v>0.028</v>
+      </c>
+      <c r="F10" s="16" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="G10" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H10" s="12" t="n">
+        <v>0.028</v>
+      </c>
+      <c r="I10" s="12" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="J10" s="13" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="K10" s="12" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="L10" s="12" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="M10" s="13" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="N10" s="12" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="O10" s="12" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="P10" s="13" t="n">
+        <v>-0.001</v>
+      </c>
+      <c r="Q10" s="12" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="R10" s="12" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="S10" s="13" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="T10" s="12" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="U10" s="12" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="V10" s="13" t="n">
+        <v>0.015</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>Mahalaxmi Bikas Bank Ltd.</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="D11" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="F11" s="15" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="G11" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="n">
+        <v>0.028</v>
+      </c>
+      <c r="I11" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="J11" s="9" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="K11" s="8" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="L11" s="8" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="M11" s="9" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="N11" s="8" t="n">
+        <v>0.03700000000000001</v>
+      </c>
+      <c r="O11" s="8" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="P11" s="9" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="Q11" s="8" t="n">
+        <v>0.03700000000000001</v>
+      </c>
+      <c r="R11" s="8" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="S11" s="9" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="T11" s="8" t="n">
+        <v>0.043</v>
+      </c>
+      <c r="U11" s="8" t="n">
+        <v>0.0425</v>
+      </c>
+      <c r="V11" s="9" t="n">
+        <v>0.0005</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>Muktinath Bikas Bank Ltd.</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="F12" s="16" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="G12" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H12" s="12" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="I12" s="12" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="J12" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="12" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="L12" s="12" t="n">
+        <v>0.028</v>
+      </c>
+      <c r="M12" s="13" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="N12" s="12" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="O12" s="12" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="P12" s="13" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="Q12" s="12" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="R12" s="12" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="S12" s="13" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="T12" s="12" t="n">
+        <v>0.0428</v>
+      </c>
+      <c r="U12" s="12" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="V12" s="13" t="n">
+        <v>0.0108</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>Narayani Development Bank Ltd.</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="n">
+        <v>0.0475</v>
+      </c>
+      <c r="C13" s="15" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="D13" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="n">
+        <v>0.0495</v>
+      </c>
+      <c r="F13" s="8" t="n">
+        <v>0.0495</v>
+      </c>
+      <c r="G13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="8" t="n">
+        <v>0.0495</v>
+      </c>
+      <c r="I13" s="8" t="n">
+        <v>0.0495</v>
+      </c>
+      <c r="J13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="8" t="n">
+        <v>0.0515</v>
+      </c>
+      <c r="L13" s="8" t="n">
+        <v>0.0515</v>
+      </c>
+      <c r="M13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="8" t="n">
+        <v>0.0515</v>
+      </c>
+      <c r="O13" s="8" t="n">
+        <v>0.0515</v>
+      </c>
+      <c r="P13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="8" t="n">
+        <v>0.0515</v>
+      </c>
+      <c r="R13" s="8" t="n">
+        <v>0.0515</v>
+      </c>
+      <c r="S13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="T13" s="8" t="n">
+        <v>0.0515</v>
+      </c>
+      <c r="U13" s="8" t="n">
+        <v>0.0515</v>
+      </c>
+      <c r="V13" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="19" t="inlineStr">
+        <is>
+          <t>Salapa Bikas Bank Ltd.</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="C14" s="12" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="D14" s="13" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="E14" s="12" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="F14" s="12" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="G14" s="13" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="H14" s="12" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="I14" s="12" t="n">
+        <v>0.0425</v>
+      </c>
+      <c r="J14" s="13" t="n">
+        <v>0.0075</v>
+      </c>
+      <c r="K14" s="12" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="L14" s="12" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M14" s="13" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="N14" s="12" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="O14" s="12" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="P14" s="13" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="Q14" s="12" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="R14" s="12" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="S14" s="13" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="T14" s="12" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="U14" s="12" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="V14" s="13" t="n">
+        <v>0.005</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>Shangri-la Development Bank Ltd.</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="C15" s="15" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="D15" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="F15" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="G15" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="I15" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="J15" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="8" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="L15" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="M15" s="9" t="n">
+        <v>0.0025</v>
+      </c>
+      <c r="N15" s="8" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="O15" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="P15" s="9" t="n">
+        <v>0.0025</v>
+      </c>
+      <c r="Q15" s="8" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="R15" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="S15" s="9" t="n">
+        <v>0.0075</v>
+      </c>
+      <c r="T15" s="8" t="n">
+        <v>0.0428</v>
+      </c>
+      <c r="U15" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="V15" s="9" t="n">
+        <v>0.0153</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="19" t="inlineStr">
+        <is>
+          <t>Shine Resunga Development Bank Ltd.</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="D16" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E16" s="12" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="F16" s="12" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="G16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="12" t="n">
+        <v>0.0325</v>
+      </c>
+      <c r="I16" s="12" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="J16" s="13" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="K16" s="12" t="n">
+        <v>0.0325</v>
+      </c>
+      <c r="L16" s="12" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="M16" s="13" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="N16" s="12" t="n">
+        <v>0.0325</v>
+      </c>
+      <c r="O16" s="12" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="P16" s="13" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="Q16" s="12" t="n">
+        <v>0.0375</v>
+      </c>
+      <c r="R16" s="12" t="n">
+        <v>0.0325</v>
+      </c>
+      <c r="S16" s="13" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="T16" s="12" t="n">
+        <v>0.0459</v>
+      </c>
+      <c r="U16" s="12" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="V16" s="13" t="n">
+        <v>0.0109</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>Sindhu Bikash Bank Ltd.</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="C17" s="15" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="D17" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="F17" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="G17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="8" t="n">
+        <v>0.0394</v>
+      </c>
+      <c r="I17" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="J17" s="9" t="n">
+        <v>0.0119</v>
+      </c>
+      <c r="K17" s="8" t="n">
+        <v>0.0394</v>
+      </c>
+      <c r="L17" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="M17" s="9" t="n">
+        <v>0.0119</v>
+      </c>
+      <c r="N17" s="8" t="n">
+        <v>0.0394</v>
+      </c>
+      <c r="O17" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="P17" s="9" t="n">
+        <v>0.0119</v>
+      </c>
+      <c r="Q17" s="8" t="n">
+        <v>0.0394</v>
+      </c>
+      <c r="R17" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="S17" s="9" t="n">
+        <v>0.0119</v>
+      </c>
+      <c r="T17" s="8" t="n">
+        <v>0.0428</v>
+      </c>
+      <c r="U17" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="V17" s="9" t="n">
+        <v>0.0153</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>Difference = Individual rate minus Institutional rate (percentage points): green = individuals earn more, red = institutions earn more, grey = same. 'Not specified' = the bank publishes no rate for that tenure (e.g. institutional FD starting at 6 months or 1 year). Rates are the general FD rate applying to a deposit of exactly that tenure; '5 Years &amp; Above' uses the band covering 5 years.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:V17"/>
+  <mergeCells count="9">
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="A1:V1"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="T3:V3"/>
+    <mergeCell ref="E3:G3"/>
+    <mergeCell ref="K3:M3"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="N3:P3"/>
+    <mergeCell ref="Q3:S3"/>
+  </mergeCells>
+  <conditionalFormatting sqref="D5:D17">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>AND(ISNUMBER(D5),D5&gt;0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="1">
+      <formula>AND(ISNUMBER(D5),D5&lt;0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="2">
+      <formula>AND(ISNUMBER(D5),D5=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G5:G17">
+    <cfRule type="expression" priority="4" dxfId="0">
+      <formula>AND(ISNUMBER(G5),G5&gt;0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" dxfId="1">
+      <formula>AND(ISNUMBER(G5),G5&lt;0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="2">
+      <formula>AND(ISNUMBER(G5),G5=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J5:J17">
+    <cfRule type="expression" priority="7" dxfId="0">
+      <formula>AND(ISNUMBER(J5),J5&gt;0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="8" dxfId="1">
+      <formula>AND(ISNUMBER(J5),J5&lt;0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="9" dxfId="2">
+      <formula>AND(ISNUMBER(J5),J5=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M5:M17">
+    <cfRule type="expression" priority="10" dxfId="0">
+      <formula>AND(ISNUMBER(M5),M5&gt;0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="11" dxfId="1">
+      <formula>AND(ISNUMBER(M5),M5&lt;0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="12" dxfId="2">
+      <formula>AND(ISNUMBER(M5),M5=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P5:P17">
+    <cfRule type="expression" priority="13" dxfId="0">
+      <formula>AND(ISNUMBER(P5),P5&gt;0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="14" dxfId="1">
+      <formula>AND(ISNUMBER(P5),P5&lt;0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="15" dxfId="2">
+      <formula>AND(ISNUMBER(P5),P5=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S5:S17">
+    <cfRule type="expression" priority="16" dxfId="0">
+      <formula>AND(ISNUMBER(S5),S5&gt;0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="17" dxfId="1">
+      <formula>AND(ISNUMBER(S5),S5&lt;0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="18" dxfId="2">
+      <formula>AND(ISNUMBER(S5),S5=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="V5:V17">
+    <cfRule type="expression" priority="19" dxfId="0">
+      <formula>AND(ISNUMBER(V5),V5&gt;0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="20" dxfId="1">
+      <formula>AND(ISNUMBER(V5),V5&lt;0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="21" dxfId="2">
+      <formula>AND(ISNUMBER(V5),V5=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:N67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -7962,7 +9251,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8006,42 +9295,42 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="18" t="inlineStr">
+      <c r="A2" s="20" t="inlineStr">
         <is>
           <t>All banks</t>
         </is>
       </c>
-      <c r="B2" s="18" t="inlineStr"/>
-      <c r="C2" s="18" t="inlineStr"/>
-      <c r="D2" s="18" t="inlineStr"/>
-      <c r="E2" s="18" t="inlineStr">
+      <c r="B2" s="20" t="inlineStr"/>
+      <c r="C2" s="20" t="inlineStr"/>
+      <c r="D2" s="20" t="inlineStr"/>
+      <c r="E2" s="20" t="inlineStr">
         <is>
           <t>Saving Max is the second highest saving rate, excluding the first highest. Call and FCY accounts are excluded from saving rates; loan, base and spread rates are excluded. Remittance FD rates are excluded from Individual FD. Months follow the Nepali calendar (Shrawan to Ashadh).</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="18" t="inlineStr">
+      <c r="A3" s="20" t="inlineStr">
         <is>
           <t>Corporate Development Bank Ltd.</t>
         </is>
       </c>
-      <c r="B3" s="18" t="inlineStr">
+      <c r="B3" s="20" t="inlineStr">
         <is>
           <t>Development Banks</t>
         </is>
       </c>
-      <c r="C3" s="18" t="inlineStr">
+      <c r="C3" s="20" t="inlineStr">
         <is>
           <t>1 Ashwin 2083 (17 Sep 2026)</t>
         </is>
       </c>
-      <c r="D3" s="18" t="inlineStr">
+      <c r="D3" s="20" t="inlineStr">
         <is>
           <t>https://merolagani.com/AnnouncementDetail.aspx?id=67425</t>
         </is>
       </c>
-      <c r="E3" s="18" t="inlineStr">
+      <c r="E3" s="20" t="inlineStr">
         <is>
           <t>• Individual FD: 3M 3.50%, 6-9M 3.75%, 1Y 4.25%, &gt;1-2Y 4.50%, &gt;2-3Y 5.00%, &gt;3-5Y 5.25%, &gt;5Y 5.50%.
 • Corporate (institutional) FD minimum 6 months: 6-9M 2.85%, 1Y 3.25%, &gt;5Y 4.75%.
@@ -8050,27 +9339,27 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="18" t="inlineStr">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>Garima Bikas Bank Ltd.</t>
         </is>
       </c>
-      <c r="B4" s="18" t="inlineStr">
+      <c r="B4" s="20" t="inlineStr">
         <is>
           <t>Development Banks</t>
         </is>
       </c>
-      <c r="C4" s="18" t="inlineStr">
+      <c r="C4" s="20" t="inlineStr">
         <is>
           <t>2083.06.01 (17 Sep 2026)</t>
         </is>
       </c>
-      <c r="D4" s="18" t="inlineStr">
+      <c r="D4" s="20" t="inlineStr">
         <is>
           <t>https://merolagani.com/AnnouncementDetail.aspx?id=67424</t>
         </is>
       </c>
-      <c r="E4" s="18" t="inlineStr">
+      <c r="E4" s="20" t="inlineStr">
         <is>
           <t>• Individual '3 Months to below 2 Years' 2.75% covers &lt;1Y and 1Y.
 • Institutional '6 Months to Below 3 Years' 2.75% covers &lt;1Y and 1Y.
@@ -8079,27 +9368,27 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="20" t="inlineStr">
         <is>
           <t>Green Development Bank Ltd.</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B5" s="20" t="inlineStr">
         <is>
           <t>Development Banks</t>
         </is>
       </c>
-      <c r="C5" s="18" t="inlineStr">
+      <c r="C5" s="20" t="inlineStr">
         <is>
           <t>1st Ashoj 2083</t>
         </is>
       </c>
-      <c r="D5" s="18" t="inlineStr">
+      <c r="D5" s="20" t="inlineStr">
         <is>
           <t>https://merolagani.com/AnnouncementDetail.aspx?id=67423</t>
         </is>
       </c>
-      <c r="E5" s="18" t="inlineStr">
+      <c r="E5" s="20" t="inlineStr">
         <is>
           <t>• FD bands: 3 Month, 6 Month, 1 Year to below 2 years, 2 to below 4 years, 4 years and above.
 • Institutional 3 Month shown as '-'; 6 Month 2.75% used as &lt;1Y max.</t>
@@ -8107,27 +9396,27 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="18" t="inlineStr">
+      <c r="A6" s="20" t="inlineStr">
         <is>
           <t>Jyoti Bikas Bank Ltd.</t>
         </is>
       </c>
-      <c r="B6" s="18" t="inlineStr">
+      <c r="B6" s="20" t="inlineStr">
         <is>
           <t>Development Banks</t>
         </is>
       </c>
-      <c r="C6" s="18" t="inlineStr">
+      <c r="C6" s="20" t="inlineStr">
         <is>
           <t>Ashwin 01, 2083 (17 Sep 2026)</t>
         </is>
       </c>
-      <c r="D6" s="18" t="inlineStr">
+      <c r="D6" s="20" t="inlineStr">
         <is>
           <t>https://merolagani.com/AnnouncementDetail.aspx?id=67422</t>
         </is>
       </c>
-      <c r="E6" s="18" t="inlineStr">
+      <c r="E6" s="20" t="inlineStr">
         <is>
           <t>• Individual: 3M 2.75%, 6M to below 3Y 2.75%, 3-5Y 2.75%, 5Y+ 4.28%.
 • Institutional: 3M '-', all other tenures 2.75%.</t>
@@ -8135,27 +9424,27 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="18" t="inlineStr">
+      <c r="A7" s="20" t="inlineStr">
         <is>
           <t>Kamana Sewa Bikas Bank Ltd.</t>
         </is>
       </c>
-      <c r="B7" s="18" t="inlineStr">
+      <c r="B7" s="20" t="inlineStr">
         <is>
           <t>Development Banks</t>
         </is>
       </c>
-      <c r="C7" s="18" t="inlineStr">
+      <c r="C7" s="20" t="inlineStr">
         <is>
           <t>1st Ashwin 2083 (17 Sep 2026)</t>
         </is>
       </c>
-      <c r="D7" s="18" t="inlineStr">
+      <c r="D7" s="20" t="inlineStr">
         <is>
           <t>https://merolagani.com/AnnouncementDetail.aspx?id=67421</t>
         </is>
       </c>
-      <c r="E7" s="18" t="inlineStr">
+      <c r="E7" s="20" t="inlineStr">
         <is>
           <t>• Individual 3 months to below 2 years 2.75%; '1 year and below 2 years' used as 1 Year.
 • Institutional FD starts at 1 year; &lt;1Y not specified.</t>
@@ -8163,27 +9452,27 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="18" t="inlineStr">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t>Lumbini Bikas Bank Ltd.</t>
         </is>
       </c>
-      <c r="B8" s="18" t="inlineStr">
+      <c r="B8" s="20" t="inlineStr">
         <is>
           <t>Development Banks</t>
         </is>
       </c>
-      <c r="C8" s="18" t="inlineStr">
+      <c r="C8" s="20" t="inlineStr">
         <is>
           <t>Ashwin month 2083</t>
         </is>
       </c>
-      <c r="D8" s="18" t="inlineStr">
+      <c r="D8" s="20" t="inlineStr">
         <is>
           <t>https://merolagani.com/AnnouncementDetail.aspx?id=67420</t>
         </is>
       </c>
-      <c r="E8" s="18" t="inlineStr">
+      <c r="E8" s="20" t="inlineStr">
         <is>
           <t>• Individual 'Upto 1 Years' 2.80% covers &lt;1Y and 1Y. Locker deposit excluded from saving.
 • Institutional starts 'Above 1 year to 2 year' (2.75%), used as 1 Year; &lt;1Y not specified.</t>
@@ -8191,27 +9480,27 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="20" t="inlineStr">
         <is>
           <t>Mahalaxmi Bikas Bank Ltd.</t>
         </is>
       </c>
-      <c r="B9" s="18" t="inlineStr">
+      <c r="B9" s="20" t="inlineStr">
         <is>
           <t>Development Banks</t>
         </is>
       </c>
-      <c r="C9" s="18" t="inlineStr">
+      <c r="C9" s="20" t="inlineStr">
         <is>
           <t>17 Sep 2026 (1st Aswin 2083)</t>
         </is>
       </c>
-      <c r="D9" s="18" t="inlineStr">
+      <c r="D9" s="20" t="inlineStr">
         <is>
           <t>https://merolagani.com/AnnouncementDetail.aspx?id=67419</t>
         </is>
       </c>
-      <c r="E9" s="18" t="inlineStr">
+      <c r="E9" s="20" t="inlineStr">
         <is>
           <t>• FD starts at 1 year for both individual and institutional; &lt;1Y not specified.
 • In-person individual rates used (mobile app rates are 0.10% higher).
@@ -8221,27 +9510,27 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>Muktinath Bikas Bank Ltd.</t>
         </is>
       </c>
-      <c r="B10" s="18" t="inlineStr">
+      <c r="B10" s="20" t="inlineStr">
         <is>
           <t>Development Banks</t>
         </is>
       </c>
-      <c r="C10" s="18" t="inlineStr">
+      <c r="C10" s="20" t="inlineStr">
         <is>
           <t>1st Ashoj 2083</t>
         </is>
       </c>
-      <c r="D10" s="18" t="inlineStr">
+      <c r="D10" s="20" t="inlineStr">
         <is>
           <t>https://merolagani.com/AnnouncementDetail.aspx?id=67418</t>
         </is>
       </c>
-      <c r="E10" s="18" t="inlineStr">
+      <c r="E10" s="20" t="inlineStr">
         <is>
           <t>• 'All other Savings' 2.75% counted once. FCY and current accounts excluded.
 • Institutional 3M and 6M shown as '-'; &lt;1Y not specified.</t>
@@ -8249,27 +9538,27 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="inlineStr">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>Narayani Development Bank Ltd.</t>
         </is>
       </c>
-      <c r="B11" s="18" t="inlineStr">
+      <c r="B11" s="20" t="inlineStr">
         <is>
           <t>Development Banks</t>
         </is>
       </c>
-      <c r="C11" s="18" t="inlineStr">
+      <c r="C11" s="20" t="inlineStr">
         <is>
           <t>Ashwin 01, 2083 (17 Sep 2026)</t>
         </is>
       </c>
-      <c r="D11" s="18" t="inlineStr">
+      <c r="D11" s="20" t="inlineStr">
         <is>
           <t>https://merolagani.com/AnnouncementDetail.aspx?id=67417</t>
         </is>
       </c>
-      <c r="E11" s="18" t="inlineStr">
+      <c r="E11" s="20" t="inlineStr">
         <is>
           <t>• Individual FD: 3-6M 4.75%, 6-12M 4.95%, 12M above 5.15%.
 • Institutional FD: 3-6M N/A, 6-12M 4.95%, 12M above 5.15% (12M above used as 1 Year).</t>
@@ -8277,54 +9566,54 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>Salapa Bikas Bank Ltd.</t>
         </is>
       </c>
-      <c r="B12" s="18" t="inlineStr">
+      <c r="B12" s="20" t="inlineStr">
         <is>
           <t>Development Banks</t>
         </is>
       </c>
-      <c r="C12" s="18" t="inlineStr">
+      <c r="C12" s="20" t="inlineStr">
         <is>
           <t>Ashoj 01, 2083</t>
         </is>
       </c>
-      <c r="D12" s="18" t="inlineStr">
+      <c r="D12" s="20" t="inlineStr">
         <is>
           <t>https://merolagani.com/AnnouncementDetail.aspx?id=67416</t>
         </is>
       </c>
-      <c r="E12" s="18" t="inlineStr">
+      <c r="E12" s="20" t="inlineStr">
         <is>
           <t>• FD bands: 3-9 months, One year, Two year and above.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="inlineStr">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>Shangri-la Development Bank Ltd.</t>
         </is>
       </c>
-      <c r="B13" s="18" t="inlineStr">
+      <c r="B13" s="20" t="inlineStr">
         <is>
           <t>Development Banks</t>
         </is>
       </c>
-      <c r="C13" s="18" t="inlineStr">
+      <c r="C13" s="20" t="inlineStr">
         <is>
           <t>Ashwin 01, 2083 (17 Sep 2026)</t>
         </is>
       </c>
-      <c r="D13" s="18" t="inlineStr">
+      <c r="D13" s="20" t="inlineStr">
         <is>
           <t>https://merolagani.com/AnnouncementDetail.aspx?id=67415</t>
         </is>
       </c>
-      <c r="E13" s="18" t="inlineStr">
+      <c r="E13" s="20" t="inlineStr">
         <is>
           <t>• Individual '3 Months to 1 Year' 2.75% covers both &lt;1Y and 1Y.
 • Institutional: single rate '6 Months and Above' 2.75% applied to all tenures.</t>
@@ -8332,54 +9621,54 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>Shine Resunga Development Bank Ltd.</t>
         </is>
       </c>
-      <c r="B14" s="18" t="inlineStr">
+      <c r="B14" s="20" t="inlineStr">
         <is>
           <t>Development Banks</t>
         </is>
       </c>
-      <c r="C14" s="18" t="inlineStr">
+      <c r="C14" s="20" t="inlineStr">
         <is>
           <t>2083-06-01 (17 Sep 2026)</t>
         </is>
       </c>
-      <c r="D14" s="18" t="inlineStr">
+      <c r="D14" s="20" t="inlineStr">
         <is>
           <t>https://merolagani.com/AnnouncementDetail.aspx?id=67414</t>
         </is>
       </c>
-      <c r="E14" s="18" t="inlineStr">
+      <c r="E14" s="20" t="inlineStr">
         <is>
           <t>• Institutional 2.75% is a single rate for 6 months to below 4 years.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>Sindhu Bikash Bank Ltd.</t>
         </is>
       </c>
-      <c r="B15" s="18" t="inlineStr">
+      <c r="B15" s="20" t="inlineStr">
         <is>
           <t>Development Banks</t>
         </is>
       </c>
-      <c r="C15" s="18" t="inlineStr">
+      <c r="C15" s="20" t="inlineStr">
         <is>
           <t>2083/06/01 (Nepali notice)</t>
         </is>
       </c>
-      <c r="D15" s="18" t="inlineStr">
+      <c r="D15" s="20" t="inlineStr">
         <is>
           <t>https://merolagani.com/AnnouncementDetail.aspx?id=67413</t>
         </is>
       </c>
-      <c r="E15" s="18" t="inlineStr">
+      <c r="E15" s="20" t="inlineStr">
         <is>
           <t>• Notice in Nepali. Margin account and current account (0.00%) excluded from saving.
 • Individual '1 year to below 5 years' 3.94% used as 1 Year.
@@ -8388,27 +9677,27 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="18" t="inlineStr">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>Agricultural Development Bank Ltd.</t>
         </is>
       </c>
-      <c r="B16" s="18" t="inlineStr">
+      <c r="B16" s="20" t="inlineStr">
         <is>
           <t>Commercial Banks</t>
         </is>
       </c>
-      <c r="C16" s="18" t="inlineStr">
+      <c r="C16" s="20" t="inlineStr">
         <is>
           <t>Aswin 01, 2083 (17 Sep 2026)</t>
         </is>
       </c>
-      <c r="D16" s="18" t="inlineStr">
+      <c r="D16" s="20" t="inlineStr">
         <is>
           <t>https://merolagani.com/AnnouncementDetail.aspx?id=67446</t>
         </is>
       </c>
-      <c r="E16" s="18" t="inlineStr">
+      <c r="E16" s="20" t="inlineStr">
         <is>
           <t>• General FD used; 'Three Months to One Year' 2.77% covers &lt;1Y and 1Y.
 • FCY saving (USD/EUR/GBP) excluded. Special FD products excluded.
@@ -8417,27 +9706,27 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="18" t="inlineStr">
+      <c r="A17" s="20" t="inlineStr">
         <is>
           <t>Citizens Bank International Ltd.</t>
         </is>
       </c>
-      <c r="B17" s="18" t="inlineStr">
+      <c r="B17" s="20" t="inlineStr">
         <is>
           <t>Commercial Banks</t>
         </is>
       </c>
-      <c r="C17" s="18" t="inlineStr">
+      <c r="C17" s="20" t="inlineStr">
         <is>
           <t>1 Ashwin 2083 (17 Sep 2026)</t>
         </is>
       </c>
-      <c r="D17" s="18" t="inlineStr">
+      <c r="D17" s="20" t="inlineStr">
         <is>
           <t>https://merolagani.com/AnnouncementDetail.aspx?id=67445</t>
         </is>
       </c>
-      <c r="E17" s="18" t="inlineStr">
+      <c r="E17" s="20" t="inlineStr">
         <is>
           <t>• Institutional FD only listed for '24 Months and above' (2.75%); &lt;1Y and 1Y not specified.
 • Individual 1 Year = '12 Months and below 24 Months' 2.90%.</t>
@@ -8445,27 +9734,27 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="18" t="inlineStr">
+      <c r="A18" s="20" t="inlineStr">
         <is>
           <t>Everest Bank Ltd.</t>
         </is>
       </c>
-      <c r="B18" s="18" t="inlineStr">
+      <c r="B18" s="20" t="inlineStr">
         <is>
           <t>Commercial Banks</t>
         </is>
       </c>
-      <c r="C18" s="18" t="inlineStr">
+      <c r="C18" s="20" t="inlineStr">
         <is>
           <t>17 Sep 2026 (1 Ashoj 2083)</t>
         </is>
       </c>
-      <c r="D18" s="18" t="inlineStr">
+      <c r="D18" s="20" t="inlineStr">
         <is>
           <t>https://merolagani.com/AnnouncementDetail.aspx?id=67385</t>
         </is>
       </c>
-      <c r="E18" s="18" t="inlineStr">
+      <c r="E18" s="20" t="inlineStr">
         <is>
           <t>• Individual 'Above 3 years' corrected from 3.50% to 3.75% per EBL correction notice (17 Sep 2026).
 • '3 months upto 3 years' 2.75% covers &lt;1Y and 1Y.</t>
@@ -8473,27 +9762,27 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="18" t="inlineStr">
+      <c r="A19" s="20" t="inlineStr">
         <is>
           <t>Global IME Bank Ltd.</t>
         </is>
       </c>
-      <c r="B19" s="18" t="inlineStr">
+      <c r="B19" s="20" t="inlineStr">
         <is>
           <t>Commercial Banks</t>
         </is>
       </c>
-      <c r="C19" s="18" t="inlineStr">
+      <c r="C19" s="20" t="inlineStr">
         <is>
           <t>Ashwin 01, 2083 (17 Sep 2026)</t>
         </is>
       </c>
-      <c r="D19" s="18" t="inlineStr">
+      <c r="D19" s="20" t="inlineStr">
         <is>
           <t>https://merolagani.com/AnnouncementDetail.aspx?id=67443</t>
         </is>
       </c>
-      <c r="E19" s="18" t="inlineStr">
+      <c r="E19" s="20" t="inlineStr">
         <is>
           <t>• Individual '3 Months to 1 Year' 2.76% used for &lt;1Y and 1Y ('Above 1 Year to below 2 Years' is 2.80%).
 • Institutional only 'Above 1 Year' 2.75%, used for 1Y and &gt;1Y; &lt;1Y not specified.</t>
@@ -8501,27 +9790,27 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="18" t="inlineStr">
+      <c r="A20" s="20" t="inlineStr">
         <is>
           <t>Himalayan Bank Ltd.</t>
         </is>
       </c>
-      <c r="B20" s="18" t="inlineStr">
+      <c r="B20" s="20" t="inlineStr">
         <is>
           <t>Commercial Banks</t>
         </is>
       </c>
-      <c r="C20" s="18" t="inlineStr">
+      <c r="C20" s="20" t="inlineStr">
         <is>
           <t>Ashwin 01, 2083 (17 Sep 2026)</t>
         </is>
       </c>
-      <c r="D20" s="18" t="inlineStr">
+      <c r="D20" s="20" t="inlineStr">
         <is>
           <t>https://merolagani.com/AnnouncementDetail.aspx?id=67442</t>
         </is>
       </c>
-      <c r="E20" s="18" t="inlineStr">
+      <c r="E20" s="20" t="inlineStr">
         <is>
           <t>• This notice only revises USD FD and fixed-rate loans; it states other deposit rates 'remain as it is'.
 • NPR saving/call/FD rates are not in the notice (see HBL's earlier notice or website).</t>
@@ -8529,27 +9818,27 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="18" t="inlineStr">
+      <c r="A21" s="20" t="inlineStr">
         <is>
           <t>Kumari Bank Ltd.</t>
         </is>
       </c>
-      <c r="B21" s="18" t="inlineStr">
+      <c r="B21" s="20" t="inlineStr">
         <is>
           <t>Commercial Banks</t>
         </is>
       </c>
-      <c r="C21" s="18" t="inlineStr">
+      <c r="C21" s="20" t="inlineStr">
         <is>
           <t>01 Ashwin 2083 (17 Sep 2026)</t>
         </is>
       </c>
-      <c r="D21" s="18" t="inlineStr">
+      <c r="D21" s="20" t="inlineStr">
         <is>
           <t>https://merolagani.com/AnnouncementDetail.aspx?id=67441</t>
         </is>
       </c>
-      <c r="E21" s="18" t="inlineStr">
+      <c r="E21" s="20" t="inlineStr">
         <is>
           <t>• In-person individual FD rates used; Kumari Smart app rates are higher (2.80% / 3.73%).
 • '3 Months to below 2 Years' 2.75% covers &lt;1Y and 1Y.</t>
@@ -8557,81 +9846,81 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="18" t="inlineStr">
+      <c r="A22" s="20" t="inlineStr">
         <is>
           <t>Laxmi Sunrise Bank Ltd.</t>
         </is>
       </c>
-      <c r="B22" s="18" t="inlineStr">
+      <c r="B22" s="20" t="inlineStr">
         <is>
           <t>Commercial Banks</t>
         </is>
       </c>
-      <c r="C22" s="18" t="inlineStr">
+      <c r="C22" s="20" t="inlineStr">
         <is>
           <t>17 Sep 2026</t>
         </is>
       </c>
-      <c r="D22" s="18" t="inlineStr">
+      <c r="D22" s="20" t="inlineStr">
         <is>
           <t>https://merolagani.com/AnnouncementDetail.aspx?id=67440</t>
         </is>
       </c>
-      <c r="E22" s="18" t="inlineStr">
+      <c r="E22" s="20" t="inlineStr">
         <is>
           <t>• 'Personal' term deposit used as Individual FD.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="18" t="inlineStr">
+      <c r="A23" s="20" t="inlineStr">
         <is>
           <t>Machhapuchchhre Bank Ltd.</t>
         </is>
       </c>
-      <c r="B23" s="18" t="inlineStr">
+      <c r="B23" s="20" t="inlineStr">
         <is>
           <t>Commercial Banks</t>
         </is>
       </c>
-      <c r="C23" s="18" t="inlineStr">
+      <c r="C23" s="20" t="inlineStr">
         <is>
           <t>17 Sep 2026</t>
         </is>
       </c>
-      <c r="D23" s="18" t="inlineStr">
+      <c r="D23" s="20" t="inlineStr">
         <is>
           <t>https://merolagani.com/AnnouncementDetail.aspx?id=67439</t>
         </is>
       </c>
-      <c r="E23" s="18" t="inlineStr">
+      <c r="E23" s="20" t="inlineStr">
         <is>
           <t>• Individual '6 months to below 3 years' 3.00% covers &lt;1Y and 1Y. Recurring deposit excluded from saving.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="18" t="inlineStr">
+      <c r="A24" s="20" t="inlineStr">
         <is>
           <t>Nabil Bank Ltd.</t>
         </is>
       </c>
-      <c r="B24" s="18" t="inlineStr">
+      <c r="B24" s="20" t="inlineStr">
         <is>
           <t>Commercial Banks</t>
         </is>
       </c>
-      <c r="C24" s="18" t="inlineStr">
+      <c r="C24" s="20" t="inlineStr">
         <is>
           <t>17 Sep 2026 (1 Ashwin 2083)</t>
         </is>
       </c>
-      <c r="D24" s="18" t="inlineStr">
+      <c r="D24" s="20" t="inlineStr">
         <is>
           <t>https://merolagani.com/AnnouncementDetail.aspx?id=67438</t>
         </is>
       </c>
-      <c r="E24" s="18" t="inlineStr">
+      <c r="E24" s="20" t="inlineStr">
         <is>
           <t>• NPR call rate not published; notice says call deposit rate is as per agreement.
 • Individual '6 months to 1 year' 2.85% used as 1 Year ('Above 1 to 2 years' is 3.00%).</t>
@@ -8639,189 +9928,189 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="18" t="inlineStr">
+      <c r="A25" s="20" t="inlineStr">
         <is>
           <t>Nepal Bank Ltd.</t>
         </is>
       </c>
-      <c r="B25" s="18" t="inlineStr">
+      <c r="B25" s="20" t="inlineStr">
         <is>
           <t>Commercial Banks</t>
         </is>
       </c>
-      <c r="C25" s="18" t="inlineStr">
+      <c r="C25" s="20" t="inlineStr">
         <is>
           <t>1st Ashwin 2083</t>
         </is>
       </c>
-      <c r="D25" s="18" t="inlineStr">
+      <c r="D25" s="20" t="inlineStr">
         <is>
           <t>https://merolagani.com/AnnouncementDetail.aspx?id=67437</t>
         </is>
       </c>
-      <c r="E25" s="18" t="inlineStr">
+      <c r="E25" s="20" t="inlineStr">
         <is>
           <t>• Individual '3M upto 1Y' 2.76% used for &lt;1Y and 1Y ('Above 1Y upto 2Y' is 3.00%).</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="18" t="inlineStr">
+      <c r="A26" s="20" t="inlineStr">
         <is>
           <t>NIC Asia Bank Ltd.</t>
         </is>
       </c>
-      <c r="B26" s="18" t="inlineStr">
+      <c r="B26" s="20" t="inlineStr">
         <is>
           <t>Commercial Banks</t>
         </is>
       </c>
-      <c r="C26" s="18" t="inlineStr">
+      <c r="C26" s="20" t="inlineStr">
         <is>
           <t>1st Ashwin 2083 (17 Sep 2026)</t>
         </is>
       </c>
-      <c r="D26" s="18" t="inlineStr">
+      <c r="D26" s="20" t="inlineStr">
         <is>
           <t>https://merolagani.com/AnnouncementDetail.aspx?id=67436</t>
         </is>
       </c>
-      <c r="E26" s="18" t="inlineStr">
+      <c r="E26" s="20" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="18" t="inlineStr">
+      <c r="A27" s="20" t="inlineStr">
         <is>
           <t>Nepal Investment Mega Bank Ltd.</t>
         </is>
       </c>
-      <c r="B27" s="18" t="inlineStr">
+      <c r="B27" s="20" t="inlineStr">
         <is>
           <t>Commercial Banks</t>
         </is>
       </c>
-      <c r="C27" s="18" t="inlineStr">
+      <c r="C27" s="20" t="inlineStr">
         <is>
           <t>17 Sep 2026 (1st Ashwin 2083)</t>
         </is>
       </c>
-      <c r="D27" s="18" t="inlineStr">
+      <c r="D27" s="20" t="inlineStr">
         <is>
           <t>https://merolagani.com/AnnouncementDetail.aspx?id=67435</t>
         </is>
       </c>
-      <c r="E27" s="18" t="inlineStr">
+      <c r="E27" s="20" t="inlineStr">
         <is>
           <t>• Institutional FD starts at 1 year; &lt;1Y not specified.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="18" t="inlineStr">
+      <c r="A28" s="20" t="inlineStr">
         <is>
           <t>NMB Bank Ltd.</t>
         </is>
       </c>
-      <c r="B28" s="18" t="inlineStr">
+      <c r="B28" s="20" t="inlineStr">
         <is>
           <t>Commercial Banks</t>
         </is>
       </c>
-      <c r="C28" s="18" t="inlineStr">
+      <c r="C28" s="20" t="inlineStr">
         <is>
           <t>Asoj 1, 2083 (17 Sep 2026)</t>
         </is>
       </c>
-      <c r="D28" s="18" t="inlineStr">
+      <c r="D28" s="20" t="inlineStr">
         <is>
           <t>https://merolagani.com/AnnouncementDetail.aspx?id=67434</t>
         </is>
       </c>
-      <c r="E28" s="18" t="inlineStr">
+      <c r="E28" s="20" t="inlineStr">
         <is>
           <t>• Institutional '3 Months to Below 1 Year' shown as '-'.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="18" t="inlineStr">
+      <c r="A29" s="20" t="inlineStr">
         <is>
           <t>Prime Commercial Bank Ltd.</t>
         </is>
       </c>
-      <c r="B29" s="18" t="inlineStr">
+      <c r="B29" s="20" t="inlineStr">
         <is>
           <t>Commercial Banks</t>
         </is>
       </c>
-      <c r="C29" s="18" t="inlineStr">
+      <c r="C29" s="20" t="inlineStr">
         <is>
           <t>01st Ashwin 2083 (17 Sep 2026)</t>
         </is>
       </c>
-      <c r="D29" s="18" t="inlineStr">
+      <c r="D29" s="20" t="inlineStr">
         <is>
           <t>https://merolagani.com/AnnouncementDetail.aspx?id=67433</t>
         </is>
       </c>
-      <c r="E29" s="18" t="inlineStr">
+      <c r="E29" s="20" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="18" t="inlineStr">
+      <c r="A30" s="20" t="inlineStr">
         <is>
           <t>Prabhu Bank Ltd.</t>
         </is>
       </c>
-      <c r="B30" s="18" t="inlineStr">
+      <c r="B30" s="20" t="inlineStr">
         <is>
           <t>Commercial Banks</t>
         </is>
       </c>
-      <c r="C30" s="18" t="inlineStr">
+      <c r="C30" s="20" t="inlineStr">
         <is>
           <t>17 Sep 2026 (01 Ashwin 2083)</t>
         </is>
       </c>
-      <c r="D30" s="18" t="inlineStr">
+      <c r="D30" s="20" t="inlineStr">
         <is>
           <t>https://merolagani.com/AnnouncementDetail.aspx?id=67432</t>
         </is>
       </c>
-      <c r="E30" s="18" t="inlineStr">
+      <c r="E30" s="20" t="inlineStr">
         <is>
           <t>• Individual '6 months to 1 year' 2.75% used as 1 Year ('Above 1 year to 3 years' is 3.10%).</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="18" t="inlineStr">
+      <c r="A31" s="20" t="inlineStr">
         <is>
           <t>Rastriya Banijya Bank Ltd.</t>
         </is>
       </c>
-      <c r="B31" s="18" t="inlineStr">
+      <c r="B31" s="20" t="inlineStr">
         <is>
           <t>Commercial Banks</t>
         </is>
       </c>
-      <c r="C31" s="18" t="inlineStr">
+      <c r="C31" s="20" t="inlineStr">
         <is>
           <t>2083 Asoj 01 (17 Sep 2026)</t>
         </is>
       </c>
-      <c r="D31" s="18" t="inlineStr">
+      <c r="D31" s="20" t="inlineStr">
         <is>
           <t>https://merolagani.com/AnnouncementDetail.aspx?id=67430</t>
         </is>
       </c>
-      <c r="E31" s="18" t="inlineStr">
+      <c r="E31" s="20" t="inlineStr">
         <is>
           <t>• Notice in Nepali. General (साधारण) FD used; '1 year to 2 years' 3.15% used as 1 Year.
 • FCY saving excluded.</t>
@@ -8829,108 +10118,108 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="18" t="inlineStr">
+      <c r="A32" s="20" t="inlineStr">
         <is>
           <t>Sanima Bank Ltd.</t>
         </is>
       </c>
-      <c r="B32" s="18" t="inlineStr">
+      <c r="B32" s="20" t="inlineStr">
         <is>
           <t>Commercial Banks</t>
         </is>
       </c>
-      <c r="C32" s="18" t="inlineStr">
+      <c r="C32" s="20" t="inlineStr">
         <is>
           <t>Ashwin 1, 2083</t>
         </is>
       </c>
-      <c r="D32" s="18" t="inlineStr">
+      <c r="D32" s="20" t="inlineStr">
         <is>
           <t>https://merolagani.com/AnnouncementDetail.aspx?id=67429</t>
         </is>
       </c>
-      <c r="E32" s="18" t="inlineStr">
+      <c r="E32" s="20" t="inlineStr">
         <is>
           <t>• Individual '3 Months to 12 Months' 2.80% covers &lt;1Y and 1Y; remittance FD excluded.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="18" t="inlineStr">
+      <c r="A33" s="20" t="inlineStr">
         <is>
           <t>Nepal SBI Bank Ltd.</t>
         </is>
       </c>
-      <c r="B33" s="18" t="inlineStr">
+      <c r="B33" s="20" t="inlineStr">
         <is>
           <t>Commercial Banks</t>
         </is>
       </c>
-      <c r="C33" s="18" t="inlineStr">
+      <c r="C33" s="20" t="inlineStr">
         <is>
           <t>17 Sep 2026 (1st Ashwin 2083)</t>
         </is>
       </c>
-      <c r="D33" s="18" t="inlineStr">
+      <c r="D33" s="20" t="inlineStr">
         <is>
           <t>https://merolagani.com/AnnouncementDetail.aspx?id=67428</t>
         </is>
       </c>
-      <c r="E33" s="18" t="inlineStr">
+      <c r="E33" s="20" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="18" t="inlineStr">
+      <c r="A34" s="20" t="inlineStr">
         <is>
           <t>Siddhartha Bank Ltd.</t>
         </is>
       </c>
-      <c r="B34" s="18" t="inlineStr">
+      <c r="B34" s="20" t="inlineStr">
         <is>
           <t>Commercial Banks</t>
         </is>
       </c>
-      <c r="C34" s="18" t="inlineStr">
+      <c r="C34" s="20" t="inlineStr">
         <is>
           <t>17 Sep 2026</t>
         </is>
       </c>
-      <c r="D34" s="18" t="inlineStr">
+      <c r="D34" s="20" t="inlineStr">
         <is>
           <t>https://merolagani.com/AnnouncementDetail.aspx?id=67427</t>
         </is>
       </c>
-      <c r="E34" s="18" t="inlineStr">
+      <c r="E34" s="20" t="inlineStr">
         <is>
           <t>• Institutional FD starts at 1 year; &lt;1Y not specified.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="18" t="inlineStr">
+      <c r="A35" s="20" t="inlineStr">
         <is>
           <t>Standard Chartered Bank Nepal Ltd.</t>
         </is>
       </c>
-      <c r="B35" s="18" t="inlineStr">
+      <c r="B35" s="20" t="inlineStr">
         <is>
           <t>Commercial Banks</t>
         </is>
       </c>
-      <c r="C35" s="18" t="inlineStr">
+      <c r="C35" s="20" t="inlineStr">
         <is>
           <t>17 Sep 2026</t>
         </is>
       </c>
-      <c r="D35" s="18" t="inlineStr">
+      <c r="D35" s="20" t="inlineStr">
         <is>
           <t>https://merolagani.com/AnnouncementDetail.aspx?id=67526</t>
         </is>
       </c>
-      <c r="E35" s="18" t="inlineStr">
+      <c r="E35" s="20" t="inlineStr">
         <is>
           <t>• Latest SCB notice (22 Sep 2026) only amends FCY FD rates; NPR rates taken from SCB's 16 Sep notice.
 • Non-individual FD: '1 year and above' 2.75%.</t>

</xml_diff>

<commit_message>
Call rate: where no direct rate is published, use 'Up to' 50% of lowest saving rate
</commit_message>
<xml_diff>
--- a/reports/Interest_Rate_Summary.xlsx
+++ b/reports/Interest_Rate_Summary.xlsx
@@ -1428,18 +1428,16 @@
       </c>
       <c r="H12" s="10" t="inlineStr">
         <is>
-          <t>As per NRB guidelines</t>
+          <t>Up to 1.375%</t>
         </is>
       </c>
       <c r="I12" s="10" t="inlineStr">
         <is>
-          <t>As per NRB guidelines</t>
-        </is>
-      </c>
-      <c r="J12" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Up to 1.375%</t>
+        </is>
+      </c>
+      <c r="J12" s="9" t="n">
+        <v>0</v>
       </c>
       <c r="K12" s="15" t="inlineStr">
         <is>
@@ -2242,18 +2240,16 @@
       </c>
       <c r="H21" s="14" t="inlineStr">
         <is>
-          <t>Negotiable as per NRB Directive</t>
+          <t>Up to 1.375%</t>
         </is>
       </c>
       <c r="I21" s="14" t="inlineStr">
         <is>
-          <t>Negotiable as per NRB Directive</t>
-        </is>
-      </c>
-      <c r="J21" s="16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Up to 1.375%</t>
+        </is>
+      </c>
+      <c r="J21" s="13" t="n">
+        <v>0</v>
       </c>
       <c r="K21" s="12" t="n">
         <v>0.0285</v>
@@ -2440,18 +2436,16 @@
       </c>
       <c r="H23" s="14" t="inlineStr">
         <is>
-          <t>Up to 50% of minimum saving deposit rate</t>
+          <t>Up to 1.375%</t>
         </is>
       </c>
       <c r="I23" s="14" t="inlineStr">
         <is>
-          <t>Up to 50% of minimum saving deposit rate</t>
-        </is>
-      </c>
-      <c r="J23" s="16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Up to 1.375%</t>
+        </is>
+      </c>
+      <c r="J23" s="13" t="n">
+        <v>0</v>
       </c>
       <c r="K23" s="12" t="n">
         <v>0.0276</v>
@@ -2774,18 +2768,16 @@
       </c>
       <c r="H26" s="10" t="inlineStr">
         <is>
-          <t>Negotiable (max 50% of lowest saving rate)</t>
+          <t>Up to 1.375%</t>
         </is>
       </c>
       <c r="I26" s="10" t="inlineStr">
         <is>
-          <t>Negotiable (max 50% of lowest saving rate)</t>
-        </is>
-      </c>
-      <c r="J26" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Up to 1.375%</t>
+        </is>
+      </c>
+      <c r="J26" s="9" t="n">
+        <v>0</v>
       </c>
       <c r="K26" s="8" t="n">
         <v>0.029</v>
@@ -2960,18 +2952,16 @@
       </c>
       <c r="H28" s="10" t="inlineStr">
         <is>
-          <t>As per agreement</t>
+          <t>Up to 1.375%</t>
         </is>
       </c>
       <c r="I28" s="10" t="inlineStr">
         <is>
-          <t>As per agreement</t>
-        </is>
-      </c>
-      <c r="J28" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Up to 1.375%</t>
+        </is>
+      </c>
+      <c r="J28" s="9" t="n">
+        <v>0</v>
       </c>
       <c r="K28" s="8" t="n">
         <v>0.0285</v>
@@ -6276,7 +6266,7 @@
       </c>
       <c r="G14" s="10" t="inlineStr">
         <is>
-          <t>As per NRB guidelines</t>
+          <t>Up to 1.375%</t>
         </is>
       </c>
       <c r="H14" s="15" t="inlineStr">
@@ -6334,7 +6324,7 @@
       </c>
       <c r="G15" s="14" t="inlineStr">
         <is>
-          <t>As per NRB guidelines</t>
+          <t>Up to 1.375%</t>
         </is>
       </c>
       <c r="H15" s="16" t="inlineStr">
@@ -7162,7 +7152,7 @@
       </c>
       <c r="G30" s="10" t="inlineStr">
         <is>
-          <t>Negotiable as per NRB Directive</t>
+          <t>Up to 1.375%</t>
         </is>
       </c>
       <c r="H30" s="8" t="n">
@@ -7220,7 +7210,7 @@
       </c>
       <c r="G31" s="14" t="inlineStr">
         <is>
-          <t>Negotiable as per NRB Directive</t>
+          <t>Up to 1.375%</t>
         </is>
       </c>
       <c r="H31" s="12" t="n">
@@ -7386,7 +7376,7 @@
       </c>
       <c r="G34" s="10" t="inlineStr">
         <is>
-          <t>Up to 50% of minimum saving deposit rate</t>
+          <t>Up to 1.375%</t>
         </is>
       </c>
       <c r="H34" s="8" t="n">
@@ -7442,7 +7432,7 @@
       </c>
       <c r="G35" s="14" t="inlineStr">
         <is>
-          <t>Up to 50% of minimum saving deposit rate</t>
+          <t>Up to 1.375%</t>
         </is>
       </c>
       <c r="H35" s="12" t="n">
@@ -7746,7 +7736,7 @@
       </c>
       <c r="G40" s="10" t="inlineStr">
         <is>
-          <t>Negotiable (max 50% of lowest saving rate)</t>
+          <t>Up to 1.375%</t>
         </is>
       </c>
       <c r="H40" s="8" t="n">
@@ -7800,7 +7790,7 @@
       </c>
       <c r="G41" s="14" t="inlineStr">
         <is>
-          <t>Negotiable (max 50% of lowest saving rate)</t>
+          <t>Up to 1.375%</t>
         </is>
       </c>
       <c r="H41" s="12" t="n">
@@ -8180,7 +8170,7 @@
       </c>
       <c r="G48" s="10" t="inlineStr">
         <is>
-          <t>As per agreement</t>
+          <t>Up to 1.375%</t>
         </is>
       </c>
       <c r="H48" s="8" t="n">
@@ -8234,7 +8224,7 @@
       </c>
       <c r="G49" s="14" t="inlineStr">
         <is>
-          <t>As per agreement</t>
+          <t>Up to 1.375%</t>
         </is>
       </c>
       <c r="H49" s="12" t="n">
@@ -9305,7 +9295,7 @@
       <c r="D2" s="20" t="inlineStr"/>
       <c r="E2" s="20" t="inlineStr">
         <is>
-          <t>Saving Max is the second highest saving rate, excluding the first highest. Call and FCY accounts are excluded from saving rates; loan, base and spread rates are excluded. Remittance FD rates are excluded from Individual FD. Months follow the Nepali calendar (Shrawan to Ashadh).</t>
+          <t>Saving Max is the second highest saving rate, excluding the first highest. Call and FCY accounts are excluded from saving rates; loan, base and spread rates are excluded. Remittance FD rates are excluded from Individual FD. Where no direct call rate is published (negotiable / as per agreement / 50% of saving rate), Call = 'Up to' 50% of the lowest saving rate. Months follow the Nepali calendar (Shrawan to Ashadh).</t>
         </is>
       </c>
     </row>
@@ -9505,7 +9495,8 @@
           <t>• FD starts at 1 year for both individual and institutional; &lt;1Y not specified.
 • In-person individual rates used (mobile app rates are 0.10% higher).
 • Dollar account, margin locker and PMS accounts excluded from saving.
-• No call rate published; notice says call deposit rate is as per NRB guidelines.</t>
+• No call rate published; notice says call deposit rate is as per NRB guidelines.
+• Call: notice says 'As per NRB guidelines'; shown as 50% of lowest saving rate (2.75%) = Up to 1.375%.</t>
         </is>
       </c>
     </row>
@@ -9729,7 +9720,8 @@
       <c r="E17" s="20" t="inlineStr">
         <is>
           <t>• Institutional FD only listed for '24 Months and above' (2.75%); &lt;1Y and 1Y not specified.
-• Individual 1 Year = '12 Months and below 24 Months' 2.90%.</t>
+• Individual 1 Year = '12 Months and below 24 Months' 2.90%.
+• Call: notice says 'Negotiable as per NRB Directive'; shown as 50% of lowest saving rate (2.75%) = Up to 1.375%.</t>
         </is>
       </c>
     </row>
@@ -9785,7 +9777,8 @@
       <c r="E19" s="20" t="inlineStr">
         <is>
           <t>• Individual '3 Months to 1 Year' 2.76% used for &lt;1Y and 1Y ('Above 1 Year to below 2 Years' is 2.80%).
-• Institutional only 'Above 1 Year' 2.75%, used for 1Y and &gt;1Y; &lt;1Y not specified.</t>
+• Institutional only 'Above 1 Year' 2.75%, used for 1Y and &gt;1Y; &lt;1Y not specified.
+• Call: notice says 'Up to 50% of minimum saving deposit rate'; shown as 50% of lowest saving rate (2.75%) = Up to 1.375%.</t>
         </is>
       </c>
     </row>
@@ -9868,7 +9861,8 @@
       </c>
       <c r="E22" s="20" t="inlineStr">
         <is>
-          <t>• 'Personal' term deposit used as Individual FD.</t>
+          <t>• 'Personal' term deposit used as Individual FD.
+• Call: notice says 'Negotiable (max 50% of lowest saving rate)'; shown as 50% of lowest saving rate (2.75%) = Up to 1.375%.</t>
         </is>
       </c>
     </row>
@@ -9923,7 +9917,8 @@
       <c r="E24" s="20" t="inlineStr">
         <is>
           <t>• NPR call rate not published; notice says call deposit rate is as per agreement.
-• Individual '6 months to 1 year' 2.85% used as 1 Year ('Above 1 to 2 years' is 3.00%).</t>
+• Individual '6 months to 1 year' 2.85% used as 1 Year ('Above 1 to 2 years' is 3.00%).
+• Call: notice says 'As per agreement'; shown as 50% of lowest saving rate (2.75%) = Up to 1.375%.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Development FD Spread: show the same 8 selected development banks
</commit_message>
<xml_diff>
--- a/reports/Interest_Rate_Summary.xlsx
+++ b/reports/Interest_Rate_Summary.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Interest Rate Summary'!$A$4:$AB$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Development FD Spread'!$A$4:$V$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Development FD Spread'!$A$4:$V$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Monthly History'!$A$1:$N$67</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3698,7 +3698,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V19"/>
+  <dimension ref="A1:V14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -3899,81 +3899,81 @@
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>Corporate Development Bank Ltd.</t>
+          <t>Garima Bikas Bank Ltd.</t>
         </is>
       </c>
       <c r="B5" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="G5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="I5" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="J5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="8" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="L5" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="M5" s="9" t="n">
+        <v>0.0025</v>
+      </c>
+      <c r="N5" s="8" t="n">
         <v>0.035</v>
       </c>
-      <c r="C5" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="D5" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="n">
-        <v>0.0375</v>
-      </c>
-      <c r="F5" s="8" t="n">
-        <v>0.0285</v>
-      </c>
-      <c r="G5" s="9" t="n">
-        <v>0.008999999999999999</v>
-      </c>
-      <c r="H5" s="8" t="n">
-        <v>0.0425</v>
-      </c>
-      <c r="I5" s="8" t="n">
+      <c r="O5" s="8" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="P5" s="9" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="Q5" s="8" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="R5" s="8" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="S5" s="9" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="T5" s="8" t="n">
+        <v>0.0428</v>
+      </c>
+      <c r="U5" s="8" t="n">
         <v>0.0325</v>
       </c>
-      <c r="J5" s="9" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="K5" s="8" t="n">
-        <v>0.045</v>
-      </c>
-      <c r="L5" s="8" t="n">
-        <v>0.035</v>
-      </c>
-      <c r="M5" s="9" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="N5" s="8" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="O5" s="8" t="n">
-        <v>0.0425</v>
-      </c>
-      <c r="P5" s="9" t="n">
-        <v>0.0075</v>
-      </c>
-      <c r="Q5" s="8" t="n">
-        <v>0.0525</v>
-      </c>
-      <c r="R5" s="8" t="n">
-        <v>0.045</v>
-      </c>
-      <c r="S5" s="9" t="n">
-        <v>0.0075</v>
-      </c>
-      <c r="T5" s="8" t="n">
-        <v>0.055</v>
-      </c>
-      <c r="U5" s="8" t="n">
-        <v>0.0475</v>
-      </c>
       <c r="V5" s="9" t="n">
-        <v>0.0075</v>
+        <v>0.0103</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="13" t="inlineStr">
         <is>
-          <t>Garima Bikas Bank Ltd.</t>
+          <t>Jyoti Bikas Bank Ltd.</t>
         </is>
       </c>
       <c r="B6" s="8" t="n">
@@ -4008,124 +4008,128 @@
         <v>0</v>
       </c>
       <c r="K6" s="8" t="n">
-        <v>0.03</v>
+        <v>0.0275</v>
       </c>
       <c r="L6" s="8" t="n">
         <v>0.0275</v>
       </c>
       <c r="M6" s="9" t="n">
-        <v>0.0025</v>
+        <v>0</v>
       </c>
       <c r="N6" s="8" t="n">
-        <v>0.035</v>
+        <v>0.0275</v>
       </c>
       <c r="O6" s="8" t="n">
-        <v>0.03</v>
+        <v>0.0275</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>0.005</v>
+        <v>0</v>
       </c>
       <c r="Q6" s="8" t="n">
-        <v>0.035</v>
+        <v>0.0275</v>
       </c>
       <c r="R6" s="8" t="n">
-        <v>0.03</v>
+        <v>0.0275</v>
       </c>
       <c r="S6" s="9" t="n">
-        <v>0.005</v>
+        <v>0</v>
       </c>
       <c r="T6" s="8" t="n">
         <v>0.0428</v>
       </c>
       <c r="U6" s="8" t="n">
-        <v>0.0325</v>
+        <v>0.0275</v>
       </c>
       <c r="V6" s="9" t="n">
-        <v>0.0103</v>
+        <v>0.0153</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="13" t="inlineStr">
         <is>
-          <t>Green Development Bank Ltd.</t>
+          <t>Kamana Sewa Bikas Bank Ltd.</t>
         </is>
       </c>
       <c r="B7" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="I7" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="J7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="8" t="n">
         <v>0.03</v>
       </c>
-      <c r="C7" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="D7" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E7" s="8" t="n">
-        <v>0.035</v>
-      </c>
-      <c r="F7" s="8" t="n">
-        <v>0.0275</v>
-      </c>
-      <c r="G7" s="9" t="n">
-        <v>0.0075</v>
-      </c>
-      <c r="H7" s="8" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="I7" s="8" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="J7" s="9" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="K7" s="8" t="n">
-        <v>0.0475</v>
-      </c>
       <c r="L7" s="8" t="n">
-        <v>0.0375</v>
+        <v>0.0275</v>
       </c>
       <c r="M7" s="9" t="n">
-        <v>0.01</v>
+        <v>0.0025</v>
       </c>
       <c r="N7" s="8" t="n">
-        <v>0.0475</v>
+        <v>0.0315</v>
       </c>
       <c r="O7" s="8" t="n">
-        <v>0.0375</v>
+        <v>0.0275</v>
       </c>
       <c r="P7" s="9" t="n">
-        <v>0.01</v>
+        <v>0.004</v>
       </c>
       <c r="Q7" s="8" t="n">
-        <v>0.0525</v>
+        <v>0.0315</v>
       </c>
       <c r="R7" s="8" t="n">
-        <v>0.0425</v>
+        <v>0.0335</v>
       </c>
       <c r="S7" s="9" t="n">
-        <v>0.01</v>
+        <v>-0.002</v>
       </c>
       <c r="T7" s="8" t="n">
-        <v>0.0525</v>
+        <v>0.0428</v>
       </c>
       <c r="U7" s="8" t="n">
-        <v>0.0425</v>
+        <v>0.0335</v>
       </c>
       <c r="V7" s="9" t="n">
-        <v>0.01</v>
+        <v>0.009299999999999999</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="13" t="inlineStr">
         <is>
-          <t>Jyoti Bikas Bank Ltd.</t>
+          <t>Lumbini Bikas Bank Ltd.</t>
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.028</v>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
@@ -4138,68 +4142,74 @@
         </is>
       </c>
       <c r="E8" s="8" t="n">
-        <v>0.0275</v>
-      </c>
-      <c r="F8" s="8" t="n">
-        <v>0.0275</v>
-      </c>
-      <c r="G8" s="9" t="n">
-        <v>0</v>
+        <v>0.028</v>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="H8" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.028</v>
       </c>
       <c r="I8" s="8" t="n">
         <v>0.0275</v>
       </c>
       <c r="J8" s="9" t="n">
-        <v>0</v>
+        <v>0.0005</v>
       </c>
       <c r="K8" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.029</v>
       </c>
       <c r="L8" s="8" t="n">
         <v>0.0275</v>
       </c>
       <c r="M8" s="9" t="n">
-        <v>0</v>
+        <v>0.0015</v>
       </c>
       <c r="N8" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.029</v>
       </c>
       <c r="O8" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.03</v>
       </c>
       <c r="P8" s="9" t="n">
-        <v>0</v>
+        <v>-0.001</v>
       </c>
       <c r="Q8" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.034</v>
       </c>
       <c r="R8" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.03</v>
       </c>
       <c r="S8" s="9" t="n">
-        <v>0</v>
+        <v>0.004</v>
       </c>
       <c r="T8" s="8" t="n">
-        <v>0.0428</v>
+        <v>0.045</v>
       </c>
       <c r="U8" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.03</v>
       </c>
       <c r="V8" s="9" t="n">
-        <v>0.0153</v>
+        <v>0.015</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="13" t="inlineStr">
         <is>
-          <t>Kamana Sewa Bikas Bank Ltd.</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="n">
-        <v>0.0275</v>
+          <t>Mahalaxmi Bikas Bank Ltd.</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
@@ -4211,8 +4221,10 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E9" s="8" t="n">
-        <v>0.0275</v>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
       </c>
       <c r="F9" s="11" t="inlineStr">
         <is>
@@ -4225,139 +4237,137 @@
         </is>
       </c>
       <c r="H9" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.028</v>
       </c>
       <c r="I9" s="8" t="n">
         <v>0.0275</v>
       </c>
       <c r="J9" s="9" t="n">
-        <v>0</v>
+        <v>0.0005</v>
       </c>
       <c r="K9" s="8" t="n">
-        <v>0.03</v>
+        <v>0.032</v>
       </c>
       <c r="L9" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.029</v>
       </c>
       <c r="M9" s="9" t="n">
-        <v>0.0025</v>
+        <v>0.003</v>
       </c>
       <c r="N9" s="8" t="n">
-        <v>0.0315</v>
+        <v>0.03700000000000001</v>
       </c>
       <c r="O9" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.032</v>
       </c>
       <c r="P9" s="9" t="n">
-        <v>0.004</v>
+        <v>0.005</v>
       </c>
       <c r="Q9" s="8" t="n">
-        <v>0.0315</v>
+        <v>0.03700000000000001</v>
       </c>
       <c r="R9" s="8" t="n">
-        <v>0.0335</v>
+        <v>0.032</v>
       </c>
       <c r="S9" s="9" t="n">
-        <v>-0.002</v>
+        <v>0.005</v>
       </c>
       <c r="T9" s="8" t="n">
-        <v>0.0428</v>
+        <v>0.043</v>
       </c>
       <c r="U9" s="8" t="n">
-        <v>0.0335</v>
+        <v>0.0425</v>
       </c>
       <c r="V9" s="9" t="n">
-        <v>0.009299999999999999</v>
+        <v>0.0005</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="13" t="inlineStr">
         <is>
-          <t>Lumbini Bikas Bank Ltd.</t>
+          <t>Muktinath Bikas Bank Ltd.</t>
         </is>
       </c>
       <c r="B10" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="I10" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="J10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="8" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="L10" s="8" t="n">
         <v>0.028</v>
       </c>
-      <c r="C10" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="D10" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="n">
-        <v>0.028</v>
-      </c>
-      <c r="F10" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="G10" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H10" s="8" t="n">
-        <v>0.028</v>
-      </c>
-      <c r="I10" s="8" t="n">
-        <v>0.0275</v>
-      </c>
-      <c r="J10" s="9" t="n">
-        <v>0.0005</v>
-      </c>
-      <c r="K10" s="8" t="n">
-        <v>0.029</v>
-      </c>
-      <c r="L10" s="8" t="n">
-        <v>0.0275</v>
-      </c>
       <c r="M10" s="9" t="n">
-        <v>0.0015</v>
+        <v>0.002</v>
       </c>
       <c r="N10" s="8" t="n">
-        <v>0.029</v>
+        <v>0.035</v>
       </c>
       <c r="O10" s="8" t="n">
         <v>0.03</v>
       </c>
       <c r="P10" s="9" t="n">
-        <v>-0.001</v>
+        <v>0.005</v>
       </c>
       <c r="Q10" s="8" t="n">
-        <v>0.034</v>
+        <v>0.035</v>
       </c>
       <c r="R10" s="8" t="n">
         <v>0.03</v>
       </c>
       <c r="S10" s="9" t="n">
-        <v>0.004</v>
+        <v>0.005</v>
       </c>
       <c r="T10" s="8" t="n">
-        <v>0.045</v>
+        <v>0.0428</v>
       </c>
       <c r="U10" s="8" t="n">
-        <v>0.03</v>
+        <v>0.032</v>
       </c>
       <c r="V10" s="9" t="n">
-        <v>0.015</v>
+        <v>0.0108</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t>Mahalaxmi Bikas Bank Ltd.</t>
-        </is>
-      </c>
-      <c r="B11" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
+          <t>Shangri-la Development Bank Ltd.</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="n">
+        <v>0.0275</v>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
@@ -4369,75 +4379,71 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E11" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="F11" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="G11" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E11" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="F11" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="G11" s="9" t="n">
+        <v>0</v>
       </c>
       <c r="H11" s="8" t="n">
-        <v>0.028</v>
+        <v>0.0275</v>
       </c>
       <c r="I11" s="8" t="n">
         <v>0.0275</v>
       </c>
       <c r="J11" s="9" t="n">
-        <v>0.0005</v>
+        <v>0</v>
       </c>
       <c r="K11" s="8" t="n">
-        <v>0.032</v>
+        <v>0.03</v>
       </c>
       <c r="L11" s="8" t="n">
-        <v>0.029</v>
+        <v>0.0275</v>
       </c>
       <c r="M11" s="9" t="n">
-        <v>0.003</v>
+        <v>0.0025</v>
       </c>
       <c r="N11" s="8" t="n">
-        <v>0.03700000000000001</v>
+        <v>0.03</v>
       </c>
       <c r="O11" s="8" t="n">
-        <v>0.032</v>
+        <v>0.0275</v>
       </c>
       <c r="P11" s="9" t="n">
-        <v>0.005</v>
+        <v>0.0025</v>
       </c>
       <c r="Q11" s="8" t="n">
-        <v>0.03700000000000001</v>
+        <v>0.035</v>
       </c>
       <c r="R11" s="8" t="n">
-        <v>0.032</v>
+        <v>0.0275</v>
       </c>
       <c r="S11" s="9" t="n">
-        <v>0.005</v>
+        <v>0.0075</v>
       </c>
       <c r="T11" s="8" t="n">
-        <v>0.043</v>
+        <v>0.0428</v>
       </c>
       <c r="U11" s="8" t="n">
-        <v>0.0425</v>
+        <v>0.0275</v>
       </c>
       <c r="V11" s="9" t="n">
-        <v>0.0005</v>
+        <v>0.0153</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="13" t="inlineStr">
         <is>
-          <t>Muktinath Bikas Bank Ltd.</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="n">
-        <v>0.0275</v>
+          <t>Shine Resunga Development Bank Ltd.</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
@@ -4452,439 +4458,67 @@
       <c r="E12" s="8" t="n">
         <v>0.0275</v>
       </c>
-      <c r="F12" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="G12" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="F12" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="G12" s="9" t="n">
+        <v>0</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.0325</v>
       </c>
       <c r="I12" s="8" t="n">
         <v>0.0275</v>
       </c>
       <c r="J12" s="9" t="n">
-        <v>0</v>
+        <v>0.005</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>0.03</v>
+        <v>0.0325</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>0.028</v>
+        <v>0.0275</v>
       </c>
       <c r="M12" s="9" t="n">
-        <v>0.002</v>
+        <v>0.005</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>0.035</v>
+        <v>0.0325</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>0.03</v>
+        <v>0.0275</v>
       </c>
       <c r="P12" s="9" t="n">
         <v>0.005</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>0.035</v>
+        <v>0.0375</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>0.03</v>
+        <v>0.0325</v>
       </c>
       <c r="S12" s="9" t="n">
         <v>0.005</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>0.0428</v>
+        <v>0.0459</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>0.032</v>
+        <v>0.035</v>
       </c>
       <c r="V12" s="9" t="n">
-        <v>0.0108</v>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="13" t="inlineStr">
-        <is>
-          <t>Narayani Development Bank Ltd.</t>
-        </is>
-      </c>
-      <c r="B13" s="8" t="n">
-        <v>0.0475</v>
-      </c>
-      <c r="C13" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="D13" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="n">
-        <v>0.0495</v>
-      </c>
-      <c r="F13" s="8" t="n">
-        <v>0.0495</v>
-      </c>
-      <c r="G13" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="8" t="n">
-        <v>0.0495</v>
-      </c>
-      <c r="I13" s="8" t="n">
-        <v>0.0495</v>
-      </c>
-      <c r="J13" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" s="8" t="n">
-        <v>0.0515</v>
-      </c>
-      <c r="L13" s="8" t="n">
-        <v>0.0515</v>
-      </c>
-      <c r="M13" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" s="8" t="n">
-        <v>0.0515</v>
-      </c>
-      <c r="O13" s="8" t="n">
-        <v>0.0515</v>
-      </c>
-      <c r="P13" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q13" s="8" t="n">
-        <v>0.0515</v>
-      </c>
-      <c r="R13" s="8" t="n">
-        <v>0.0515</v>
-      </c>
-      <c r="S13" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="T13" s="8" t="n">
-        <v>0.0515</v>
-      </c>
-      <c r="U13" s="8" t="n">
-        <v>0.0515</v>
-      </c>
-      <c r="V13" s="9" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="13" t="inlineStr">
-        <is>
-          <t>Salapa Bikas Bank Ltd.</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="n">
-        <v>0.045</v>
-      </c>
-      <c r="C14" s="8" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="D14" s="9" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="E14" s="8" t="n">
-        <v>0.045</v>
-      </c>
-      <c r="F14" s="8" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="G14" s="9" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="H14" s="8" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="I14" s="8" t="n">
-        <v>0.0425</v>
-      </c>
-      <c r="J14" s="9" t="n">
-        <v>0.0075</v>
-      </c>
-      <c r="K14" s="8" t="n">
-        <v>0.055</v>
-      </c>
-      <c r="L14" s="8" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="M14" s="9" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="N14" s="8" t="n">
-        <v>0.055</v>
-      </c>
-      <c r="O14" s="8" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="P14" s="9" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="Q14" s="8" t="n">
-        <v>0.055</v>
-      </c>
-      <c r="R14" s="8" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="S14" s="9" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="T14" s="8" t="n">
-        <v>0.055</v>
-      </c>
-      <c r="U14" s="8" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="V14" s="9" t="n">
-        <v>0.005</v>
-      </c>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="13" t="inlineStr">
-        <is>
-          <t>Shangri-la Development Bank Ltd.</t>
-        </is>
-      </c>
-      <c r="B15" s="8" t="n">
-        <v>0.0275</v>
-      </c>
-      <c r="C15" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="D15" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="n">
-        <v>0.0275</v>
-      </c>
-      <c r="F15" s="8" t="n">
-        <v>0.0275</v>
-      </c>
-      <c r="G15" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" s="8" t="n">
-        <v>0.0275</v>
-      </c>
-      <c r="I15" s="8" t="n">
-        <v>0.0275</v>
-      </c>
-      <c r="J15" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" s="8" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="L15" s="8" t="n">
-        <v>0.0275</v>
-      </c>
-      <c r="M15" s="9" t="n">
-        <v>0.0025</v>
-      </c>
-      <c r="N15" s="8" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="O15" s="8" t="n">
-        <v>0.0275</v>
-      </c>
-      <c r="P15" s="9" t="n">
-        <v>0.0025</v>
-      </c>
-      <c r="Q15" s="8" t="n">
-        <v>0.035</v>
-      </c>
-      <c r="R15" s="8" t="n">
-        <v>0.0275</v>
-      </c>
-      <c r="S15" s="9" t="n">
-        <v>0.0075</v>
-      </c>
-      <c r="T15" s="8" t="n">
-        <v>0.0428</v>
-      </c>
-      <c r="U15" s="8" t="n">
-        <v>0.0275</v>
-      </c>
-      <c r="V15" s="9" t="n">
-        <v>0.0153</v>
-      </c>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="13" t="inlineStr">
-        <is>
-          <t>Shine Resunga Development Bank Ltd.</t>
-        </is>
-      </c>
-      <c r="B16" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="C16" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="D16" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="n">
-        <v>0.0275</v>
-      </c>
-      <c r="F16" s="8" t="n">
-        <v>0.0275</v>
-      </c>
-      <c r="G16" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="8" t="n">
-        <v>0.0325</v>
-      </c>
-      <c r="I16" s="8" t="n">
-        <v>0.0275</v>
-      </c>
-      <c r="J16" s="9" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="K16" s="8" t="n">
-        <v>0.0325</v>
-      </c>
-      <c r="L16" s="8" t="n">
-        <v>0.0275</v>
-      </c>
-      <c r="M16" s="9" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="N16" s="8" t="n">
-        <v>0.0325</v>
-      </c>
-      <c r="O16" s="8" t="n">
-        <v>0.0275</v>
-      </c>
-      <c r="P16" s="9" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="Q16" s="8" t="n">
-        <v>0.0375</v>
-      </c>
-      <c r="R16" s="8" t="n">
-        <v>0.0325</v>
-      </c>
-      <c r="S16" s="9" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="T16" s="8" t="n">
-        <v>0.0459</v>
-      </c>
-      <c r="U16" s="8" t="n">
-        <v>0.035</v>
-      </c>
-      <c r="V16" s="9" t="n">
         <v>0.0109</v>
       </c>
     </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="13" t="inlineStr">
-        <is>
-          <t>Sindhu Bikash Bank Ltd.</t>
-        </is>
-      </c>
-      <c r="B17" s="8" t="n">
-        <v>0.0275</v>
-      </c>
-      <c r="C17" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="D17" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="n">
-        <v>0.0275</v>
-      </c>
-      <c r="F17" s="8" t="n">
-        <v>0.0275</v>
-      </c>
-      <c r="G17" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" s="8" t="n">
-        <v>0.0394</v>
-      </c>
-      <c r="I17" s="8" t="n">
-        <v>0.0275</v>
-      </c>
-      <c r="J17" s="9" t="n">
-        <v>0.0119</v>
-      </c>
-      <c r="K17" s="8" t="n">
-        <v>0.0394</v>
-      </c>
-      <c r="L17" s="8" t="n">
-        <v>0.0275</v>
-      </c>
-      <c r="M17" s="9" t="n">
-        <v>0.0119</v>
-      </c>
-      <c r="N17" s="8" t="n">
-        <v>0.0394</v>
-      </c>
-      <c r="O17" s="8" t="n">
-        <v>0.0275</v>
-      </c>
-      <c r="P17" s="9" t="n">
-        <v>0.0119</v>
-      </c>
-      <c r="Q17" s="8" t="n">
-        <v>0.0394</v>
-      </c>
-      <c r="R17" s="8" t="n">
-        <v>0.0275</v>
-      </c>
-      <c r="S17" s="9" t="n">
-        <v>0.0119</v>
-      </c>
-      <c r="T17" s="8" t="n">
-        <v>0.0428</v>
-      </c>
-      <c r="U17" s="8" t="n">
-        <v>0.0275</v>
-      </c>
-      <c r="V17" s="9" t="n">
-        <v>0.0153</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="12" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>Difference = Individual rate minus Institutional rate (percentage points): green = individuals earn more, red = institutions earn more, grey = same. 'Not specified' = the bank publishes no rate for that tenure (e.g. institutional FD starting at 6 months or 1 year). Rates are the general FD rate applying to a deposit of exactly that tenure; '5 Years &amp; Above' uses the band covering 5 years.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:V17"/>
+  <autoFilter ref="A4:V12"/>
   <mergeCells count="9">
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="A1:V1"/>
@@ -4896,7 +4530,7 @@
     <mergeCell ref="N3:P3"/>
     <mergeCell ref="Q3:S3"/>
   </mergeCells>
-  <conditionalFormatting sqref="D5:D17">
+  <conditionalFormatting sqref="D5:D12">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>AND(ISNUMBER(D5),D5&gt;0)</formula>
     </cfRule>
@@ -4907,7 +4541,7 @@
       <formula>AND(ISNUMBER(D5),D5=0)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G5:G17">
+  <conditionalFormatting sqref="G5:G12">
     <cfRule type="expression" priority="4" dxfId="0">
       <formula>AND(ISNUMBER(G5),G5&gt;0)</formula>
     </cfRule>
@@ -4918,7 +4552,7 @@
       <formula>AND(ISNUMBER(G5),G5=0)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J5:J17">
+  <conditionalFormatting sqref="J5:J12">
     <cfRule type="expression" priority="7" dxfId="0">
       <formula>AND(ISNUMBER(J5),J5&gt;0)</formula>
     </cfRule>
@@ -4929,7 +4563,7 @@
       <formula>AND(ISNUMBER(J5),J5=0)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M5:M17">
+  <conditionalFormatting sqref="M5:M12">
     <cfRule type="expression" priority="10" dxfId="0">
       <formula>AND(ISNUMBER(M5),M5&gt;0)</formula>
     </cfRule>
@@ -4940,7 +4574,7 @@
       <formula>AND(ISNUMBER(M5),M5=0)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P5:P17">
+  <conditionalFormatting sqref="P5:P12">
     <cfRule type="expression" priority="13" dxfId="0">
       <formula>AND(ISNUMBER(P5),P5&gt;0)</formula>
     </cfRule>
@@ -4951,7 +4585,7 @@
       <formula>AND(ISNUMBER(P5),P5=0)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S5:S17">
+  <conditionalFormatting sqref="S5:S12">
     <cfRule type="expression" priority="16" dxfId="0">
       <formula>AND(ISNUMBER(S5),S5&gt;0)</formula>
     </cfRule>
@@ -4962,7 +4596,7 @@
       <formula>AND(ISNUMBER(S5),S5=0)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V5:V17">
+  <conditionalFormatting sqref="V5:V12">
     <cfRule type="expression" priority="19" dxfId="0">
       <formula>AND(ISNUMBER(V5),V5&gt;0)</formula>
     </cfRule>

</xml_diff>

<commit_message>
Report: drop Notes sheet; Monthly History limited to last 12 months
</commit_message>
<xml_diff>
--- a/reports/Interest_Rate_Summary.xlsx
+++ b/reports/Interest_Rate_Summary.xlsx
@@ -10,7 +10,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interest Rate Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development FD Spread" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly History" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Interest Rate Summary'!$A$4:$AB$34</definedName>
@@ -111,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -142,9 +141,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -8364,848 +8360,4 @@
   <autoFilter ref="A1:N67"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E30"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="100" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Bank</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>Sector</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Effective Date</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Source Document</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>Notes (Ashwin 2083)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="14" t="inlineStr">
-        <is>
-          <t>All banks</t>
-        </is>
-      </c>
-      <c r="B2" s="14" t="inlineStr"/>
-      <c r="C2" s="14" t="inlineStr"/>
-      <c r="D2" s="14" t="inlineStr"/>
-      <c r="E2" s="14" t="inlineStr">
-        <is>
-          <t>Saving Max is the second highest saving rate, excluding the first highest. Call and FCY accounts are excluded from saving rates; loan, base and spread rates are excluded. Remittance FD rates are excluded from Individual FD. Where no direct call rate is published (negotiable / as per agreement / 50% of saving rate), Call = 'Up to' 50% of the lowest saving rate. Months follow the Nepali calendar (Shrawan to Ashadh).</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>Garima Bikas Bank Ltd.</t>
-        </is>
-      </c>
-      <c r="B3" s="14" t="inlineStr">
-        <is>
-          <t>Development Banks</t>
-        </is>
-      </c>
-      <c r="C3" s="14" t="inlineStr">
-        <is>
-          <t>2083.06.01 (17 Sep 2026)</t>
-        </is>
-      </c>
-      <c r="D3" s="14" t="inlineStr">
-        <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67424</t>
-        </is>
-      </c>
-      <c r="E3" s="14" t="inlineStr">
-        <is>
-          <t>• Individual '3 Months to below 2 Years' 2.75% covers &lt;1Y and 1Y.
-• Institutional '6 Months to Below 3 Years' 2.75% covers &lt;1Y and 1Y.
-• Current, margin and FCY saving accounts excluded from saving.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="14" t="inlineStr">
-        <is>
-          <t>Jyoti Bikas Bank Ltd.</t>
-        </is>
-      </c>
-      <c r="B4" s="14" t="inlineStr">
-        <is>
-          <t>Development Banks</t>
-        </is>
-      </c>
-      <c r="C4" s="14" t="inlineStr">
-        <is>
-          <t>Ashwin 01, 2083 (17 Sep 2026)</t>
-        </is>
-      </c>
-      <c r="D4" s="14" t="inlineStr">
-        <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67422</t>
-        </is>
-      </c>
-      <c r="E4" s="14" t="inlineStr">
-        <is>
-          <t>• Individual: 3M 2.75%, 6M to below 3Y 2.75%, 3-5Y 2.75%, 5Y+ 4.28%.
-• Institutional: 3M '-', all other tenures 2.75%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="14" t="inlineStr">
-        <is>
-          <t>Kamana Sewa Bikas Bank Ltd.</t>
-        </is>
-      </c>
-      <c r="B5" s="14" t="inlineStr">
-        <is>
-          <t>Development Banks</t>
-        </is>
-      </c>
-      <c r="C5" s="14" t="inlineStr">
-        <is>
-          <t>1st Ashwin 2083 (17 Sep 2026)</t>
-        </is>
-      </c>
-      <c r="D5" s="14" t="inlineStr">
-        <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67421</t>
-        </is>
-      </c>
-      <c r="E5" s="14" t="inlineStr">
-        <is>
-          <t>• Individual 3 months to below 2 years 2.75%; '1 year and below 2 years' used as 1 Year.
-• Institutional FD starts at 1 year; &lt;1Y not specified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="14" t="inlineStr">
-        <is>
-          <t>Lumbini Bikas Bank Ltd.</t>
-        </is>
-      </c>
-      <c r="B6" s="14" t="inlineStr">
-        <is>
-          <t>Development Banks</t>
-        </is>
-      </c>
-      <c r="C6" s="14" t="inlineStr">
-        <is>
-          <t>Ashwin month 2083</t>
-        </is>
-      </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67420</t>
-        </is>
-      </c>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>• Individual 'Upto 1 Years' 2.80% covers &lt;1Y and 1Y. Locker deposit excluded from saving.
-• Institutional starts 'Above 1 year to 2 year' (2.75%), used as 1 Year; &lt;1Y not specified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="14" t="inlineStr">
-        <is>
-          <t>Mahalaxmi Bikas Bank Ltd.</t>
-        </is>
-      </c>
-      <c r="B7" s="14" t="inlineStr">
-        <is>
-          <t>Development Banks</t>
-        </is>
-      </c>
-      <c r="C7" s="14" t="inlineStr">
-        <is>
-          <t>17 Sep 2026 (1st Aswin 2083)</t>
-        </is>
-      </c>
-      <c r="D7" s="14" t="inlineStr">
-        <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67419</t>
-        </is>
-      </c>
-      <c r="E7" s="14" t="inlineStr">
-        <is>
-          <t>• FD starts at 1 year for both individual and institutional; &lt;1Y not specified.
-• In-person individual rates used (mobile app rates are 0.10% higher).
-• Dollar account, margin locker and PMS accounts excluded from saving.
-• No call rate published; notice says call deposit rate is as per NRB guidelines.
-• Call: notice says 'As per NRB guidelines'; shown as 50% of lowest saving rate (2.75%) = Up to 1.375%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="14" t="inlineStr">
-        <is>
-          <t>Muktinath Bikas Bank Ltd.</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="inlineStr">
-        <is>
-          <t>Development Banks</t>
-        </is>
-      </c>
-      <c r="C8" s="14" t="inlineStr">
-        <is>
-          <t>1st Ashoj 2083</t>
-        </is>
-      </c>
-      <c r="D8" s="14" t="inlineStr">
-        <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67418</t>
-        </is>
-      </c>
-      <c r="E8" s="14" t="inlineStr">
-        <is>
-          <t>• 'All other Savings' 2.75% counted once. FCY and current accounts excluded.
-• Institutional 3M and 6M shown as '-'; &lt;1Y not specified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="14" t="inlineStr">
-        <is>
-          <t>Shangri-la Development Bank Ltd.</t>
-        </is>
-      </c>
-      <c r="B9" s="14" t="inlineStr">
-        <is>
-          <t>Development Banks</t>
-        </is>
-      </c>
-      <c r="C9" s="14" t="inlineStr">
-        <is>
-          <t>Ashwin 01, 2083 (17 Sep 2026)</t>
-        </is>
-      </c>
-      <c r="D9" s="14" t="inlineStr">
-        <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67415</t>
-        </is>
-      </c>
-      <c r="E9" s="14" t="inlineStr">
-        <is>
-          <t>• Individual '3 Months to 1 Year' 2.75% covers both &lt;1Y and 1Y.
-• Institutional: single rate '6 Months and Above' 2.75% applied to all tenures.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="14" t="inlineStr">
-        <is>
-          <t>Shine Resunga Development Bank Ltd.</t>
-        </is>
-      </c>
-      <c r="B10" s="14" t="inlineStr">
-        <is>
-          <t>Development Banks</t>
-        </is>
-      </c>
-      <c r="C10" s="14" t="inlineStr">
-        <is>
-          <t>2083-06-01 (17 Sep 2026)</t>
-        </is>
-      </c>
-      <c r="D10" s="14" t="inlineStr">
-        <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67414</t>
-        </is>
-      </c>
-      <c r="E10" s="14" t="inlineStr">
-        <is>
-          <t>• Institutional 2.75% is a single rate for 6 months to below 4 years.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="14" t="inlineStr">
-        <is>
-          <t>Agricultural Development Bank Ltd.</t>
-        </is>
-      </c>
-      <c r="B11" s="14" t="inlineStr">
-        <is>
-          <t>Commercial Banks</t>
-        </is>
-      </c>
-      <c r="C11" s="14" t="inlineStr">
-        <is>
-          <t>Aswin 01, 2083 (17 Sep 2026)</t>
-        </is>
-      </c>
-      <c r="D11" s="14" t="inlineStr">
-        <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67446</t>
-        </is>
-      </c>
-      <c r="E11" s="14" t="inlineStr">
-        <is>
-          <t>• General FD used; 'Three Months to One Year' 2.77% covers &lt;1Y and 1Y.
-• FCY saving (USD/EUR/GBP) excluded. Special FD products excluded.
-• Institutional: single rate 'Six Months and Above' 2.75% applied to all tenures.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="14" t="inlineStr">
-        <is>
-          <t>Citizens Bank International Ltd.</t>
-        </is>
-      </c>
-      <c r="B12" s="14" t="inlineStr">
-        <is>
-          <t>Commercial Banks</t>
-        </is>
-      </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>1 Ashwin 2083 (17 Sep 2026)</t>
-        </is>
-      </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67445</t>
-        </is>
-      </c>
-      <c r="E12" s="14" t="inlineStr">
-        <is>
-          <t>• Institutional FD only listed for '24 Months and above' (2.75%); &lt;1Y and 1Y not specified.
-• Individual 1 Year = '12 Months and below 24 Months' 2.90%.
-• Call: notice says 'Negotiable as per NRB Directive'; shown as 50% of lowest saving rate (2.75%) = Up to 1.375%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="14" t="inlineStr">
-        <is>
-          <t>Everest Bank Ltd.</t>
-        </is>
-      </c>
-      <c r="B13" s="14" t="inlineStr">
-        <is>
-          <t>Commercial Banks</t>
-        </is>
-      </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>17 Sep 2026 (1 Ashoj 2083)</t>
-        </is>
-      </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67385</t>
-        </is>
-      </c>
-      <c r="E13" s="14" t="inlineStr">
-        <is>
-          <t>• Individual 'Above 3 years' corrected from 3.50% to 3.75% per EBL correction notice (17 Sep 2026).
-• '3 months upto 3 years' 2.75% covers &lt;1Y and 1Y.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="14" t="inlineStr">
-        <is>
-          <t>Global IME Bank Ltd.</t>
-        </is>
-      </c>
-      <c r="B14" s="14" t="inlineStr">
-        <is>
-          <t>Commercial Banks</t>
-        </is>
-      </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>Ashwin 01, 2083 (17 Sep 2026)</t>
-        </is>
-      </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67443</t>
-        </is>
-      </c>
-      <c r="E14" s="14" t="inlineStr">
-        <is>
-          <t>• Individual '3 Months to 1 Year' 2.76% used for &lt;1Y and 1Y ('Above 1 Year to below 2 Years' is 2.80%).
-• Institutional only 'Above 1 Year' 2.75%, used for 1Y and &gt;1Y; &lt;1Y not specified.
-• Call: notice says 'Up to 50% of minimum saving deposit rate'; shown as 50% of lowest saving rate (2.75%) = Up to 1.375%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="14" t="inlineStr">
-        <is>
-          <t>Himalayan Bank Ltd.</t>
-        </is>
-      </c>
-      <c r="B15" s="14" t="inlineStr">
-        <is>
-          <t>Commercial Banks</t>
-        </is>
-      </c>
-      <c r="C15" s="14" t="inlineStr">
-        <is>
-          <t>Ashwin 01, 2083 (17 Sep 2026)</t>
-        </is>
-      </c>
-      <c r="D15" s="14" t="inlineStr">
-        <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67442</t>
-        </is>
-      </c>
-      <c r="E15" s="14" t="inlineStr">
-        <is>
-          <t>• This notice only revises USD FD and fixed-rate loans; it states other deposit rates 'remain as it is'.
-• NPR saving/call/FD rates are not in the notice (see HBL's earlier notice or website).</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="14" t="inlineStr">
-        <is>
-          <t>Kumari Bank Ltd.</t>
-        </is>
-      </c>
-      <c r="B16" s="14" t="inlineStr">
-        <is>
-          <t>Commercial Banks</t>
-        </is>
-      </c>
-      <c r="C16" s="14" t="inlineStr">
-        <is>
-          <t>01 Ashwin 2083 (17 Sep 2026)</t>
-        </is>
-      </c>
-      <c r="D16" s="14" t="inlineStr">
-        <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67441</t>
-        </is>
-      </c>
-      <c r="E16" s="14" t="inlineStr">
-        <is>
-          <t>• In-person individual FD rates used; Kumari Smart app rates are higher (2.80% / 3.73%).
-• '3 Months to below 2 Years' 2.75% covers &lt;1Y and 1Y.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="14" t="inlineStr">
-        <is>
-          <t>Laxmi Sunrise Bank Ltd.</t>
-        </is>
-      </c>
-      <c r="B17" s="14" t="inlineStr">
-        <is>
-          <t>Commercial Banks</t>
-        </is>
-      </c>
-      <c r="C17" s="14" t="inlineStr">
-        <is>
-          <t>17 Sep 2026</t>
-        </is>
-      </c>
-      <c r="D17" s="14" t="inlineStr">
-        <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67440</t>
-        </is>
-      </c>
-      <c r="E17" s="14" t="inlineStr">
-        <is>
-          <t>• 'Personal' term deposit used as Individual FD.
-• Call: notice says 'Negotiable (max 50% of lowest saving rate)'; shown as 50% of lowest saving rate (2.75%) = Up to 1.375%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="14" t="inlineStr">
-        <is>
-          <t>Machhapuchchhre Bank Ltd.</t>
-        </is>
-      </c>
-      <c r="B18" s="14" t="inlineStr">
-        <is>
-          <t>Commercial Banks</t>
-        </is>
-      </c>
-      <c r="C18" s="14" t="inlineStr">
-        <is>
-          <t>17 Sep 2026</t>
-        </is>
-      </c>
-      <c r="D18" s="14" t="inlineStr">
-        <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67439</t>
-        </is>
-      </c>
-      <c r="E18" s="14" t="inlineStr">
-        <is>
-          <t>• Individual '6 months to below 3 years' 3.00% covers &lt;1Y and 1Y. Recurring deposit excluded from saving.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="14" t="inlineStr">
-        <is>
-          <t>Nabil Bank Ltd.</t>
-        </is>
-      </c>
-      <c r="B19" s="14" t="inlineStr">
-        <is>
-          <t>Commercial Banks</t>
-        </is>
-      </c>
-      <c r="C19" s="14" t="inlineStr">
-        <is>
-          <t>17 Sep 2026 (1 Ashwin 2083)</t>
-        </is>
-      </c>
-      <c r="D19" s="14" t="inlineStr">
-        <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67438</t>
-        </is>
-      </c>
-      <c r="E19" s="14" t="inlineStr">
-        <is>
-          <t>• NPR call rate not published; notice says call deposit rate is as per agreement.
-• Individual '6 months to 1 year' 2.85% used as 1 Year ('Above 1 to 2 years' is 3.00%).
-• Call: notice says 'As per agreement'; shown as 50% of lowest saving rate (2.75%) = Up to 1.375%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="14" t="inlineStr">
-        <is>
-          <t>Nepal Bank Ltd.</t>
-        </is>
-      </c>
-      <c r="B20" s="14" t="inlineStr">
-        <is>
-          <t>Commercial Banks</t>
-        </is>
-      </c>
-      <c r="C20" s="14" t="inlineStr">
-        <is>
-          <t>1st Ashwin 2083</t>
-        </is>
-      </c>
-      <c r="D20" s="14" t="inlineStr">
-        <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67437</t>
-        </is>
-      </c>
-      <c r="E20" s="14" t="inlineStr">
-        <is>
-          <t>• Individual '3M upto 1Y' 2.76% used for &lt;1Y and 1Y ('Above 1Y upto 2Y' is 3.00%).</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="14" t="inlineStr">
-        <is>
-          <t>NIC Asia Bank Ltd.</t>
-        </is>
-      </c>
-      <c r="B21" s="14" t="inlineStr">
-        <is>
-          <t>Commercial Banks</t>
-        </is>
-      </c>
-      <c r="C21" s="14" t="inlineStr">
-        <is>
-          <t>1st Ashwin 2083 (17 Sep 2026)</t>
-        </is>
-      </c>
-      <c r="D21" s="14" t="inlineStr">
-        <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67436</t>
-        </is>
-      </c>
-      <c r="E21" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="14" t="inlineStr">
-        <is>
-          <t>Nepal Investment Mega Bank Ltd.</t>
-        </is>
-      </c>
-      <c r="B22" s="14" t="inlineStr">
-        <is>
-          <t>Commercial Banks</t>
-        </is>
-      </c>
-      <c r="C22" s="14" t="inlineStr">
-        <is>
-          <t>17 Sep 2026 (1st Ashwin 2083)</t>
-        </is>
-      </c>
-      <c r="D22" s="14" t="inlineStr">
-        <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67435</t>
-        </is>
-      </c>
-      <c r="E22" s="14" t="inlineStr">
-        <is>
-          <t>• Institutional FD starts at 1 year; &lt;1Y not specified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="14" t="inlineStr">
-        <is>
-          <t>NMB Bank Ltd.</t>
-        </is>
-      </c>
-      <c r="B23" s="14" t="inlineStr">
-        <is>
-          <t>Commercial Banks</t>
-        </is>
-      </c>
-      <c r="C23" s="14" t="inlineStr">
-        <is>
-          <t>Asoj 1, 2083 (17 Sep 2026)</t>
-        </is>
-      </c>
-      <c r="D23" s="14" t="inlineStr">
-        <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67434</t>
-        </is>
-      </c>
-      <c r="E23" s="14" t="inlineStr">
-        <is>
-          <t>• Institutional '3 Months to Below 1 Year' shown as '-'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="14" t="inlineStr">
-        <is>
-          <t>Prime Commercial Bank Ltd.</t>
-        </is>
-      </c>
-      <c r="B24" s="14" t="inlineStr">
-        <is>
-          <t>Commercial Banks</t>
-        </is>
-      </c>
-      <c r="C24" s="14" t="inlineStr">
-        <is>
-          <t>01st Ashwin 2083 (17 Sep 2026)</t>
-        </is>
-      </c>
-      <c r="D24" s="14" t="inlineStr">
-        <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67433</t>
-        </is>
-      </c>
-      <c r="E24" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="14" t="inlineStr">
-        <is>
-          <t>Prabhu Bank Ltd.</t>
-        </is>
-      </c>
-      <c r="B25" s="14" t="inlineStr">
-        <is>
-          <t>Commercial Banks</t>
-        </is>
-      </c>
-      <c r="C25" s="14" t="inlineStr">
-        <is>
-          <t>17 Sep 2026 (01 Ashwin 2083)</t>
-        </is>
-      </c>
-      <c r="D25" s="14" t="inlineStr">
-        <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67432</t>
-        </is>
-      </c>
-      <c r="E25" s="14" t="inlineStr">
-        <is>
-          <t>• Individual '6 months to 1 year' 2.75% used as 1 Year ('Above 1 year to 3 years' is 3.10%).</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="14" t="inlineStr">
-        <is>
-          <t>Rastriya Banijya Bank Ltd.</t>
-        </is>
-      </c>
-      <c r="B26" s="14" t="inlineStr">
-        <is>
-          <t>Commercial Banks</t>
-        </is>
-      </c>
-      <c r="C26" s="14" t="inlineStr">
-        <is>
-          <t>2083 Asoj 01 (17 Sep 2026)</t>
-        </is>
-      </c>
-      <c r="D26" s="14" t="inlineStr">
-        <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67430</t>
-        </is>
-      </c>
-      <c r="E26" s="14" t="inlineStr">
-        <is>
-          <t>• Notice in Nepali. General (साधारण) FD used; '1 year to 2 years' 3.15% used as 1 Year.
-• FCY saving excluded.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="14" t="inlineStr">
-        <is>
-          <t>Sanima Bank Ltd.</t>
-        </is>
-      </c>
-      <c r="B27" s="14" t="inlineStr">
-        <is>
-          <t>Commercial Banks</t>
-        </is>
-      </c>
-      <c r="C27" s="14" t="inlineStr">
-        <is>
-          <t>Ashwin 1, 2083</t>
-        </is>
-      </c>
-      <c r="D27" s="14" t="inlineStr">
-        <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67429</t>
-        </is>
-      </c>
-      <c r="E27" s="14" t="inlineStr">
-        <is>
-          <t>• Individual '3 Months to 12 Months' 2.80% covers &lt;1Y and 1Y; remittance FD excluded.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="14" t="inlineStr">
-        <is>
-          <t>Nepal SBI Bank Ltd.</t>
-        </is>
-      </c>
-      <c r="B28" s="14" t="inlineStr">
-        <is>
-          <t>Commercial Banks</t>
-        </is>
-      </c>
-      <c r="C28" s="14" t="inlineStr">
-        <is>
-          <t>17 Sep 2026 (1st Ashwin 2083)</t>
-        </is>
-      </c>
-      <c r="D28" s="14" t="inlineStr">
-        <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67428</t>
-        </is>
-      </c>
-      <c r="E28" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="14" t="inlineStr">
-        <is>
-          <t>Siddhartha Bank Ltd.</t>
-        </is>
-      </c>
-      <c r="B29" s="14" t="inlineStr">
-        <is>
-          <t>Commercial Banks</t>
-        </is>
-      </c>
-      <c r="C29" s="14" t="inlineStr">
-        <is>
-          <t>17 Sep 2026</t>
-        </is>
-      </c>
-      <c r="D29" s="14" t="inlineStr">
-        <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67427</t>
-        </is>
-      </c>
-      <c r="E29" s="14" t="inlineStr">
-        <is>
-          <t>• Institutional FD starts at 1 year; &lt;1Y not specified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="14" t="inlineStr">
-        <is>
-          <t>Standard Chartered Bank Nepal Ltd.</t>
-        </is>
-      </c>
-      <c r="B30" s="14" t="inlineStr">
-        <is>
-          <t>Commercial Banks</t>
-        </is>
-      </c>
-      <c r="C30" s="14" t="inlineStr">
-        <is>
-          <t>17 Sep 2026</t>
-        </is>
-      </c>
-      <c r="D30" s="14" t="inlineStr">
-        <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67526</t>
-        </is>
-      </c>
-      <c r="E30" s="14" t="inlineStr">
-        <is>
-          <t>• Latest SCB notice (22 Sep 2026) only amends FCY FD rates; NPR rates taken from SCB's 16 Sep notice.
-• Non-individual FD: '1 year and above' 2.75%.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Carry forward previous month's rates for 'unchanged' and partial notices; HBL/Sindhu Shrawan baselines
</commit_message>
<xml_diff>
--- a/reports/Interest_Rate_Summary.xlsx
+++ b/reports/Interest_Rate_Summary.xlsx
@@ -14,7 +14,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Interest Rate Summary'!$A$4:$AB$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Development FD Spread'!$A$4:$V$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Monthly History'!$A$1:$N$67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Monthly History'!$A$1:$N$69</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2001,140 +2001,90 @@
           <t>Himalayan Bank Ltd.</t>
         </is>
       </c>
-      <c r="B19" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="C19" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="D19" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E19" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="F19" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="G19" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H19" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="I19" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="J19" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K19" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="L19" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="M19" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N19" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="O19" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="P19" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q19" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="R19" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="S19" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="T19" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="U19" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="V19" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="W19" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="X19" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="Y19" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Z19" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="AA19" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="AB19" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="B19" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="C19" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="D19" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="8" t="n">
+        <v>0.0325</v>
+      </c>
+      <c r="F19" s="8" t="n">
+        <v>0.0325</v>
+      </c>
+      <c r="G19" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="10" t="inlineStr">
+        <is>
+          <t>Up to 1.375%</t>
+        </is>
+      </c>
+      <c r="I19" s="10" t="inlineStr">
+        <is>
+          <t>Up to 1.375%</t>
+        </is>
+      </c>
+      <c r="J19" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="8" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="L19" s="8" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="M19" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" s="8" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="O19" s="8" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="P19" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="8" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="R19" s="8" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="S19" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="T19" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="U19" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="V19" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="W19" s="8" t="n">
+        <v>0.0276</v>
+      </c>
+      <c r="X19" s="8" t="n">
+        <v>0.0276</v>
+      </c>
+      <c r="Y19" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z19" s="8" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="AA19" s="8" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="AB19" s="9" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
@@ -4613,7 +4563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N67"/>
+  <dimension ref="A1:N69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -6031,56 +5981,44 @@
       </c>
       <c r="C26" s="10" t="inlineStr">
         <is>
-          <t>Bhadra 2083</t>
+          <t>Shrawan 2083</t>
         </is>
       </c>
       <c r="D26" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E26" s="11" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="E26" s="8" t="n">
+        <v>0.0285</v>
+      </c>
+      <c r="F26" s="8" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="G26" s="11" t="inlineStr">
         <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="F26" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="G26" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="H26" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
+      <c r="H26" s="8" t="n">
+        <v>0.0276</v>
       </c>
       <c r="I26" s="8" t="n">
-        <v>0.0441</v>
+        <v>0.046</v>
       </c>
       <c r="J26" s="8" t="n">
-        <v>0.0441</v>
-      </c>
-      <c r="K26" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="L26" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="M26" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
+        <v>0.046</v>
+      </c>
+      <c r="K26" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="L26" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="M26" s="8" t="n">
+        <v>0.0275</v>
       </c>
       <c r="N26" s="10" t="inlineStr">
         <is>
-          <t>2083/05/01 (Nepali notice)</t>
+          <t>2083/04/01 (Nepali notice)</t>
         </is>
       </c>
     </row>
@@ -6097,31 +6035,31 @@
       </c>
       <c r="C27" s="10" t="inlineStr">
         <is>
-          <t>Ashwin 2083</t>
+          <t>Bhadra 2083</t>
         </is>
       </c>
       <c r="D27" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E27" s="8" t="n">
         <v>0.0275</v>
       </c>
       <c r="F27" s="8" t="n">
-        <v>0.028</v>
-      </c>
-      <c r="G27" s="10" t="inlineStr">
-        <is>
-          <t>Up to 1.37%</t>
+        <v>0.03</v>
+      </c>
+      <c r="G27" s="11" t="inlineStr">
+        <is>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="H27" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.0276</v>
       </c>
       <c r="I27" s="8" t="n">
-        <v>0.0394</v>
+        <v>0.0441</v>
       </c>
       <c r="J27" s="8" t="n">
-        <v>0.0428</v>
+        <v>0.0441</v>
       </c>
       <c r="K27" s="8" t="n">
         <v>0.0275</v>
@@ -6134,48 +6072,48 @@
       </c>
       <c r="N27" s="10" t="inlineStr">
         <is>
-          <t>2083/06/01 (Nepali notice)</t>
+          <t>2083/05/01 (Nepali notice)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="10" t="inlineStr">
         <is>
-          <t>Agricultural Development Bank Ltd.</t>
+          <t>Sindhu Bikash Bank Ltd.</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>Commercial Banks</t>
+          <t>Development Banks</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>Bhadra 2083</t>
+          <t>Ashwin 2083</t>
         </is>
       </c>
       <c r="D28" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E28" s="8" t="n">
-        <v>0.0278</v>
+        <v>0.0275</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>0.0339</v>
+        <v>0.028</v>
       </c>
       <c r="G28" s="10" t="inlineStr">
         <is>
-          <t>0.60%</t>
+          <t>Up to 1.37%</t>
         </is>
       </c>
       <c r="H28" s="8" t="n">
-        <v>0.0278</v>
+        <v>0.0275</v>
       </c>
       <c r="I28" s="8" t="n">
-        <v>0.0278</v>
+        <v>0.0394</v>
       </c>
       <c r="J28" s="8" t="n">
-        <v>0.0415</v>
+        <v>0.0428</v>
       </c>
       <c r="K28" s="8" t="n">
         <v>0.0275</v>
@@ -6188,7 +6126,7 @@
       </c>
       <c r="N28" s="10" t="inlineStr">
         <is>
-          <t>Bhadra 01, 2083 (17 Aug 2026)</t>
+          <t>2083/06/01 (Nepali notice)</t>
         </is>
       </c>
     </row>
@@ -6205,28 +6143,28 @@
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>Ashwin 2083</t>
+          <t>Bhadra 2083</t>
         </is>
       </c>
       <c r="D29" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E29" s="8" t="n">
-        <v>0.0277</v>
+        <v>0.0278</v>
       </c>
       <c r="F29" s="8" t="n">
-        <v>0.0304</v>
+        <v>0.0339</v>
       </c>
       <c r="G29" s="10" t="inlineStr">
         <is>
-          <t>0.45%</t>
+          <t>0.60%</t>
         </is>
       </c>
       <c r="H29" s="8" t="n">
-        <v>0.0277</v>
+        <v>0.0278</v>
       </c>
       <c r="I29" s="8" t="n">
-        <v>0.0277</v>
+        <v>0.0278</v>
       </c>
       <c r="J29" s="8" t="n">
         <v>0.0415</v>
@@ -6242,14 +6180,14 @@
       </c>
       <c r="N29" s="10" t="inlineStr">
         <is>
-          <t>Aswin 01, 2083 (17 Sep 2026)</t>
+          <t>Bhadra 01, 2083 (17 Aug 2026)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="10" t="inlineStr">
         <is>
-          <t>Citizens Bank International Ltd.</t>
+          <t>Agricultural Development Bank Ltd.</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">
@@ -6259,48 +6197,44 @@
       </c>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>Bhadra 2083</t>
+          <t>Ashwin 2083</t>
         </is>
       </c>
       <c r="D30" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E30" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.0277</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>0.028</v>
+        <v>0.0304</v>
       </c>
       <c r="G30" s="10" t="inlineStr">
         <is>
-          <t>Up to 1.375%</t>
+          <t>0.45%</t>
         </is>
       </c>
       <c r="H30" s="8" t="n">
-        <v>0.0285</v>
+        <v>0.0277</v>
       </c>
       <c r="I30" s="8" t="n">
-        <v>0.029</v>
+        <v>0.0277</v>
       </c>
       <c r="J30" s="8" t="n">
-        <v>0.0385</v>
-      </c>
-      <c r="K30" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="L30" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
+        <v>0.0415</v>
+      </c>
+      <c r="K30" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="L30" s="8" t="n">
+        <v>0.0275</v>
       </c>
       <c r="M30" s="8" t="n">
-        <v>0.03</v>
+        <v>0.0275</v>
       </c>
       <c r="N30" s="10" t="inlineStr">
         <is>
-          <t>1st Bhadra 2083 (17 Aug 2026)</t>
+          <t>Aswin 01, 2083 (17 Sep 2026)</t>
         </is>
       </c>
     </row>
@@ -6317,11 +6251,11 @@
       </c>
       <c r="C31" s="10" t="inlineStr">
         <is>
-          <t>Ashwin 2083</t>
+          <t>Bhadra 2083</t>
         </is>
       </c>
       <c r="D31" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E31" s="8" t="n">
         <v>0.0275</v>
@@ -6354,18 +6288,18 @@
         </is>
       </c>
       <c r="M31" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.03</v>
       </c>
       <c r="N31" s="10" t="inlineStr">
         <is>
-          <t>1 Ashwin 2083 (17 Sep 2026)</t>
+          <t>1st Bhadra 2083 (17 Aug 2026)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="10" t="inlineStr">
         <is>
-          <t>Everest Bank Ltd.</t>
+          <t>Citizens Bank International Ltd.</t>
         </is>
       </c>
       <c r="B32" s="10" t="inlineStr">
@@ -6375,44 +6309,48 @@
       </c>
       <c r="C32" s="10" t="inlineStr">
         <is>
-          <t>Bhadra 2083</t>
+          <t>Ashwin 2083</t>
         </is>
       </c>
       <c r="D32" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E32" s="8" t="n">
         <v>0.0275</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.028</v>
       </c>
       <c r="G32" s="10" t="inlineStr">
         <is>
-          <t>Up to 0.50%</t>
+          <t>Up to 1.375%</t>
         </is>
       </c>
       <c r="H32" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.0285</v>
       </c>
       <c r="I32" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.029</v>
       </c>
       <c r="J32" s="8" t="n">
-        <v>0.0405</v>
-      </c>
-      <c r="K32" s="8" t="n">
-        <v>0.0275</v>
-      </c>
-      <c r="L32" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.0385</v>
+      </c>
+      <c r="K32" s="11" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="L32" s="11" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
       </c>
       <c r="M32" s="8" t="n">
-        <v>0.035</v>
+        <v>0.0275</v>
       </c>
       <c r="N32" s="10" t="inlineStr">
         <is>
-          <t>17 Aug 2026 (1st Bhadra 2083)</t>
+          <t>1 Ashwin 2083 (17 Sep 2026)</t>
         </is>
       </c>
     </row>
@@ -6429,11 +6367,11 @@
       </c>
       <c r="C33" s="10" t="inlineStr">
         <is>
-          <t>Ashwin 2083</t>
+          <t>Bhadra 2083</t>
         </is>
       </c>
       <c r="D33" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E33" s="8" t="n">
         <v>0.0275</v>
@@ -6453,7 +6391,7 @@
         <v>0.0275</v>
       </c>
       <c r="J33" s="8" t="n">
-        <v>0.0375</v>
+        <v>0.0405</v>
       </c>
       <c r="K33" s="8" t="n">
         <v>0.0275</v>
@@ -6462,18 +6400,18 @@
         <v>0.0275</v>
       </c>
       <c r="M33" s="8" t="n">
-        <v>0.0325</v>
+        <v>0.035</v>
       </c>
       <c r="N33" s="10" t="inlineStr">
         <is>
-          <t>17 Sep 2026 (1 Ashoj 2083)</t>
+          <t>17 Aug 2026 (1st Bhadra 2083)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="10" t="inlineStr">
         <is>
-          <t>Global IME Bank Ltd.</t>
+          <t>Everest Bank Ltd.</t>
         </is>
       </c>
       <c r="B34" s="10" t="inlineStr">
@@ -6483,11 +6421,11 @@
       </c>
       <c r="C34" s="10" t="inlineStr">
         <is>
-          <t>Bhadra 2083</t>
+          <t>Ashwin 2083</t>
         </is>
       </c>
       <c r="D34" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E34" s="8" t="n">
         <v>0.0275</v>
@@ -6497,32 +6435,30 @@
       </c>
       <c r="G34" s="10" t="inlineStr">
         <is>
-          <t>Up to 1.375%</t>
+          <t>Up to 0.50%</t>
         </is>
       </c>
       <c r="H34" s="8" t="n">
-        <v>0.0276</v>
+        <v>0.0275</v>
       </c>
       <c r="I34" s="8" t="n">
-        <v>0.0276</v>
+        <v>0.0275</v>
       </c>
       <c r="J34" s="8" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="K34" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
+        <v>0.0375</v>
+      </c>
+      <c r="K34" s="8" t="n">
+        <v>0.0275</v>
       </c>
       <c r="L34" s="8" t="n">
         <v>0.0275</v>
       </c>
       <c r="M34" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.0325</v>
       </c>
       <c r="N34" s="10" t="inlineStr">
         <is>
-          <t>Bhadra 01, 2083 (17 Aug 2026)</t>
+          <t>17 Sep 2026 (1 Ashoj 2083)</t>
         </is>
       </c>
     </row>
@@ -6539,11 +6475,11 @@
       </c>
       <c r="C35" s="10" t="inlineStr">
         <is>
-          <t>Ashwin 2083</t>
+          <t>Bhadra 2083</t>
         </is>
       </c>
       <c r="D35" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E35" s="8" t="n">
         <v>0.0275</v>
@@ -6578,14 +6514,14 @@
       </c>
       <c r="N35" s="10" t="inlineStr">
         <is>
-          <t>Ashwin 01, 2083 (17 Sep 2026)</t>
+          <t>Bhadra 01, 2083 (17 Aug 2026)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="10" t="inlineStr">
         <is>
-          <t>Himalayan Bank Ltd.</t>
+          <t>Global IME Bank Ltd.</t>
         </is>
       </c>
       <c r="B36" s="10" t="inlineStr">
@@ -6595,60 +6531,46 @@
       </c>
       <c r="C36" s="10" t="inlineStr">
         <is>
-          <t>Bhadra 2083</t>
+          <t>Ashwin 2083</t>
         </is>
       </c>
       <c r="D36" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E36" s="11" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="E36" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="F36" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="G36" s="10" t="inlineStr">
+        <is>
+          <t>Up to 1.375%</t>
+        </is>
+      </c>
+      <c r="H36" s="8" t="n">
+        <v>0.0276</v>
+      </c>
+      <c r="I36" s="8" t="n">
+        <v>0.0276</v>
+      </c>
+      <c r="J36" s="8" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="K36" s="11" t="inlineStr">
         <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="F36" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="G36" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="H36" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="I36" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="J36" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="K36" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="L36" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="M36" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
+      <c r="L36" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="M36" s="8" t="n">
+        <v>0.0275</v>
       </c>
       <c r="N36" s="10" t="inlineStr">
         <is>
-          <t>Bhadra 2083 (Nepali notice)</t>
+          <t>Ashwin 01, 2083 (17 Sep 2026)</t>
         </is>
       </c>
     </row>
@@ -6665,67 +6587,51 @@
       </c>
       <c r="C37" s="10" t="inlineStr">
         <is>
-          <t>Ashwin 2083</t>
+          <t>Shrawan 2083</t>
         </is>
       </c>
       <c r="D37" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="E37" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="F37" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="G37" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="H37" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="I37" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="J37" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="K37" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="L37" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="M37" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="E37" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="F37" s="8" t="n">
+        <v>0.0325</v>
+      </c>
+      <c r="G37" s="10" t="inlineStr">
+        <is>
+          <t>Up to 1.375%</t>
+        </is>
+      </c>
+      <c r="H37" s="8" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="I37" s="8" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="J37" s="8" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="K37" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="L37" s="8" t="n">
+        <v>0.0276</v>
+      </c>
+      <c r="M37" s="8" t="n">
+        <v>0.035</v>
       </c>
       <c r="N37" s="10" t="inlineStr">
         <is>
-          <t>Ashwin 01, 2083 (17 Sep 2026)</t>
+          <t>Shrawan 01, 2083 (17 Jul 2026)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="10" t="inlineStr">
         <is>
-          <t>Kumari Bank Ltd.</t>
+          <t>Himalayan Bank Ltd.</t>
         </is>
       </c>
       <c r="B38" s="10" t="inlineStr">
@@ -6745,41 +6651,41 @@
         <v>0.0275</v>
       </c>
       <c r="F38" s="8" t="n">
-        <v>0.0391</v>
+        <v>0.0325</v>
       </c>
       <c r="G38" s="10" t="inlineStr">
         <is>
-          <t>Up to 0.81%</t>
+          <t>Up to 1.375%</t>
         </is>
       </c>
       <c r="H38" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.029</v>
       </c>
       <c r="I38" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.03</v>
       </c>
       <c r="J38" s="8" t="n">
-        <v>0.0346</v>
+        <v>0.04</v>
       </c>
       <c r="K38" s="8" t="n">
         <v>0.0275</v>
       </c>
       <c r="L38" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.0276</v>
       </c>
       <c r="M38" s="8" t="n">
-        <v>0.0301</v>
+        <v>0.035</v>
       </c>
       <c r="N38" s="10" t="inlineStr">
         <is>
-          <t>01 Bhadra 2083 (17 Aug 2026)</t>
+          <t>Bhadra 2083 (Nepali notice)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="10" t="inlineStr">
         <is>
-          <t>Kumari Bank Ltd.</t>
+          <t>Himalayan Bank Ltd.</t>
         </is>
       </c>
       <c r="B39" s="10" t="inlineStr">
@@ -6799,41 +6705,41 @@
         <v>0.0275</v>
       </c>
       <c r="F39" s="8" t="n">
-        <v>0.0391</v>
+        <v>0.0325</v>
       </c>
       <c r="G39" s="10" t="inlineStr">
         <is>
-          <t>Up to 0.81%</t>
+          <t>Up to 1.375%</t>
         </is>
       </c>
       <c r="H39" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.029</v>
       </c>
       <c r="I39" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.03</v>
       </c>
       <c r="J39" s="8" t="n">
-        <v>0.0343</v>
+        <v>0.04</v>
       </c>
       <c r="K39" s="8" t="n">
         <v>0.0275</v>
       </c>
       <c r="L39" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.0276</v>
       </c>
       <c r="M39" s="8" t="n">
-        <v>0.0301</v>
+        <v>0.035</v>
       </c>
       <c r="N39" s="10" t="inlineStr">
         <is>
-          <t>01 Ashwin 2083 (17 Sep 2026)</t>
+          <t>Ashwin 01, 2083 (17 Sep 2026)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="10" t="inlineStr">
         <is>
-          <t>Laxmi Sunrise Bank Ltd.</t>
+          <t>Kumari Bank Ltd.</t>
         </is>
       </c>
       <c r="B40" s="10" t="inlineStr">
@@ -6853,21 +6759,21 @@
         <v>0.0275</v>
       </c>
       <c r="F40" s="8" t="n">
-        <v>0.028</v>
+        <v>0.0391</v>
       </c>
       <c r="G40" s="10" t="inlineStr">
         <is>
-          <t>Up to 1.375%</t>
+          <t>Up to 0.81%</t>
         </is>
       </c>
       <c r="H40" s="8" t="n">
-        <v>0.029</v>
+        <v>0.0275</v>
       </c>
       <c r="I40" s="8" t="n">
-        <v>0.03</v>
+        <v>0.0275</v>
       </c>
       <c r="J40" s="8" t="n">
-        <v>0.04</v>
+        <v>0.0346</v>
       </c>
       <c r="K40" s="8" t="n">
         <v>0.0275</v>
@@ -6876,18 +6782,18 @@
         <v>0.0275</v>
       </c>
       <c r="M40" s="8" t="n">
-        <v>0.0325</v>
+        <v>0.0301</v>
       </c>
       <c r="N40" s="10" t="inlineStr">
         <is>
-          <t>17 Aug 2026</t>
+          <t>01 Bhadra 2083 (17 Aug 2026)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="10" t="inlineStr">
         <is>
-          <t>Laxmi Sunrise Bank Ltd.</t>
+          <t>Kumari Bank Ltd.</t>
         </is>
       </c>
       <c r="B41" s="10" t="inlineStr">
@@ -6907,21 +6813,21 @@
         <v>0.0275</v>
       </c>
       <c r="F41" s="8" t="n">
-        <v>0.028</v>
+        <v>0.0391</v>
       </c>
       <c r="G41" s="10" t="inlineStr">
         <is>
-          <t>Up to 1.375%</t>
+          <t>Up to 0.81%</t>
         </is>
       </c>
       <c r="H41" s="8" t="n">
-        <v>0.029</v>
+        <v>0.0275</v>
       </c>
       <c r="I41" s="8" t="n">
-        <v>0.03</v>
+        <v>0.0275</v>
       </c>
       <c r="J41" s="8" t="n">
-        <v>0.04</v>
+        <v>0.0343</v>
       </c>
       <c r="K41" s="8" t="n">
         <v>0.0275</v>
@@ -6930,18 +6836,18 @@
         <v>0.0275</v>
       </c>
       <c r="M41" s="8" t="n">
-        <v>0.0325</v>
+        <v>0.0301</v>
       </c>
       <c r="N41" s="10" t="inlineStr">
         <is>
-          <t>17 Sep 2026</t>
+          <t>01 Ashwin 2083 (17 Sep 2026)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="10" t="inlineStr">
         <is>
-          <t>Machhapuchchhre Bank Ltd.</t>
+          <t>Laxmi Sunrise Bank Ltd.</t>
         </is>
       </c>
       <c r="B42" s="10" t="inlineStr">
@@ -6958,24 +6864,24 @@
         <v>2</v>
       </c>
       <c r="E42" s="8" t="n">
-        <v>0.0276</v>
+        <v>0.0275</v>
       </c>
       <c r="F42" s="8" t="n">
-        <v>0.0301</v>
+        <v>0.028</v>
       </c>
       <c r="G42" s="10" t="inlineStr">
         <is>
-          <t>Up to 0.25%</t>
+          <t>Up to 1.375%</t>
         </is>
       </c>
       <c r="H42" s="8" t="n">
-        <v>0.03</v>
+        <v>0.029</v>
       </c>
       <c r="I42" s="8" t="n">
         <v>0.03</v>
       </c>
       <c r="J42" s="8" t="n">
-        <v>0.045</v>
+        <v>0.04</v>
       </c>
       <c r="K42" s="8" t="n">
         <v>0.0275</v>
@@ -6984,7 +6890,7 @@
         <v>0.0275</v>
       </c>
       <c r="M42" s="8" t="n">
-        <v>0.03</v>
+        <v>0.0325</v>
       </c>
       <c r="N42" s="10" t="inlineStr">
         <is>
@@ -6995,7 +6901,7 @@
     <row r="43">
       <c r="A43" s="10" t="inlineStr">
         <is>
-          <t>Machhapuchchhre Bank Ltd.</t>
+          <t>Laxmi Sunrise Bank Ltd.</t>
         </is>
       </c>
       <c r="B43" s="10" t="inlineStr">
@@ -7019,17 +6925,17 @@
       </c>
       <c r="G43" s="10" t="inlineStr">
         <is>
-          <t>Up to 0.25%</t>
+          <t>Up to 1.375%</t>
         </is>
       </c>
       <c r="H43" s="8" t="n">
-        <v>0.03</v>
+        <v>0.029</v>
       </c>
       <c r="I43" s="8" t="n">
         <v>0.03</v>
       </c>
       <c r="J43" s="8" t="n">
-        <v>0.045</v>
+        <v>0.04</v>
       </c>
       <c r="K43" s="8" t="n">
         <v>0.0275</v>
@@ -7038,7 +6944,7 @@
         <v>0.0275</v>
       </c>
       <c r="M43" s="8" t="n">
-        <v>0.03</v>
+        <v>0.0325</v>
       </c>
       <c r="N43" s="10" t="inlineStr">
         <is>
@@ -7049,7 +6955,7 @@
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>NIC Asia Bank Ltd.</t>
+          <t>Machhapuchchhre Bank Ltd.</t>
         </is>
       </c>
       <c r="B44" s="10" t="inlineStr">
@@ -7066,24 +6972,24 @@
         <v>2</v>
       </c>
       <c r="E44" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.0276</v>
       </c>
       <c r="F44" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.0301</v>
       </c>
       <c r="G44" s="10" t="inlineStr">
         <is>
-          <t>Up to 1.37%</t>
+          <t>Up to 0.25%</t>
         </is>
       </c>
       <c r="H44" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.03</v>
       </c>
       <c r="I44" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.03</v>
       </c>
       <c r="J44" s="8" t="n">
-        <v>0.04</v>
+        <v>0.045</v>
       </c>
       <c r="K44" s="8" t="n">
         <v>0.0275</v>
@@ -7096,14 +7002,14 @@
       </c>
       <c r="N44" s="10" t="inlineStr">
         <is>
-          <t>1st Bhadra 2083 (17 Aug 2026)</t>
+          <t>17 Aug 2026</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t>NIC Asia Bank Ltd.</t>
+          <t>Machhapuchchhre Bank Ltd.</t>
         </is>
       </c>
       <c r="B45" s="10" t="inlineStr">
@@ -7123,21 +7029,21 @@
         <v>0.0275</v>
       </c>
       <c r="F45" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.028</v>
       </c>
       <c r="G45" s="10" t="inlineStr">
         <is>
-          <t>Up to 1.37%</t>
+          <t>Up to 0.25%</t>
         </is>
       </c>
       <c r="H45" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.03</v>
       </c>
       <c r="I45" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.03</v>
       </c>
       <c r="J45" s="8" t="n">
-        <v>0.04</v>
+        <v>0.045</v>
       </c>
       <c r="K45" s="8" t="n">
         <v>0.0275</v>
@@ -7150,14 +7056,14 @@
       </c>
       <c r="N45" s="10" t="inlineStr">
         <is>
-          <t>1st Ashwin 2083 (17 Sep 2026)</t>
+          <t>17 Sep 2026</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="10" t="inlineStr">
         <is>
-          <t>NMB Bank Ltd.</t>
+          <t>NIC Asia Bank Ltd.</t>
         </is>
       </c>
       <c r="B46" s="10" t="inlineStr">
@@ -7181,7 +7087,7 @@
       </c>
       <c r="G46" s="10" t="inlineStr">
         <is>
-          <t>Up to 1.375%</t>
+          <t>Up to 1.37%</t>
         </is>
       </c>
       <c r="H46" s="8" t="n">
@@ -7191,7 +7097,7 @@
         <v>0.0275</v>
       </c>
       <c r="J46" s="8" t="n">
-        <v>0.045</v>
+        <v>0.04</v>
       </c>
       <c r="K46" s="8" t="n">
         <v>0.0275</v>
@@ -7200,18 +7106,18 @@
         <v>0.0275</v>
       </c>
       <c r="M46" s="8" t="n">
-        <v>0.035</v>
+        <v>0.03</v>
       </c>
       <c r="N46" s="10" t="inlineStr">
         <is>
-          <t>Bhadra 1, 2083 (17 Aug 2026)</t>
+          <t>1st Bhadra 2083 (17 Aug 2026)</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="10" t="inlineStr">
         <is>
-          <t>NMB Bank Ltd.</t>
+          <t>NIC Asia Bank Ltd.</t>
         </is>
       </c>
       <c r="B47" s="10" t="inlineStr">
@@ -7235,7 +7141,7 @@
       </c>
       <c r="G47" s="10" t="inlineStr">
         <is>
-          <t>Up to 1.375%</t>
+          <t>Up to 1.37%</t>
         </is>
       </c>
       <c r="H47" s="8" t="n">
@@ -7245,29 +7151,27 @@
         <v>0.0275</v>
       </c>
       <c r="J47" s="8" t="n">
-        <v>0.045</v>
-      </c>
-      <c r="K47" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
+        <v>0.04</v>
+      </c>
+      <c r="K47" s="8" t="n">
+        <v>0.0275</v>
       </c>
       <c r="L47" s="8" t="n">
         <v>0.0275</v>
       </c>
       <c r="M47" s="8" t="n">
-        <v>0.035</v>
+        <v>0.03</v>
       </c>
       <c r="N47" s="10" t="inlineStr">
         <is>
-          <t>Asoj 1, 2083 (17 Sep 2026)</t>
+          <t>1st Ashwin 2083 (17 Sep 2026)</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="10" t="inlineStr">
         <is>
-          <t>Nabil Bank Ltd.</t>
+          <t>NMB Bank Ltd.</t>
         </is>
       </c>
       <c r="B48" s="10" t="inlineStr">
@@ -7287,7 +7191,7 @@
         <v>0.0275</v>
       </c>
       <c r="F48" s="8" t="n">
-        <v>0.028</v>
+        <v>0.0275</v>
       </c>
       <c r="G48" s="10" t="inlineStr">
         <is>
@@ -7295,13 +7199,13 @@
         </is>
       </c>
       <c r="H48" s="8" t="n">
-        <v>0.0285</v>
+        <v>0.0275</v>
       </c>
       <c r="I48" s="8" t="n">
-        <v>0.0285</v>
+        <v>0.0275</v>
       </c>
       <c r="J48" s="8" t="n">
-        <v>0.0455</v>
+        <v>0.045</v>
       </c>
       <c r="K48" s="8" t="n">
         <v>0.0275</v>
@@ -7310,18 +7214,18 @@
         <v>0.0275</v>
       </c>
       <c r="M48" s="8" t="n">
-        <v>0.0301</v>
+        <v>0.035</v>
       </c>
       <c r="N48" s="10" t="inlineStr">
         <is>
-          <t>17 Aug 2026 (1st Bhadra 2083)</t>
+          <t>Bhadra 1, 2083 (17 Aug 2026)</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="10" t="inlineStr">
         <is>
-          <t>Nabil Bank Ltd.</t>
+          <t>NMB Bank Ltd.</t>
         </is>
       </c>
       <c r="B49" s="10" t="inlineStr">
@@ -7341,7 +7245,7 @@
         <v>0.0275</v>
       </c>
       <c r="F49" s="8" t="n">
-        <v>0.028</v>
+        <v>0.0275</v>
       </c>
       <c r="G49" s="10" t="inlineStr">
         <is>
@@ -7349,33 +7253,35 @@
         </is>
       </c>
       <c r="H49" s="8" t="n">
-        <v>0.0285</v>
+        <v>0.0275</v>
       </c>
       <c r="I49" s="8" t="n">
-        <v>0.0285</v>
+        <v>0.0275</v>
       </c>
       <c r="J49" s="8" t="n">
-        <v>0.0425</v>
-      </c>
-      <c r="K49" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.045</v>
+      </c>
+      <c r="K49" s="11" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
       </c>
       <c r="L49" s="8" t="n">
         <v>0.0275</v>
       </c>
       <c r="M49" s="8" t="n">
-        <v>0.0301</v>
+        <v>0.035</v>
       </c>
       <c r="N49" s="10" t="inlineStr">
         <is>
-          <t>17 Sep 2026 (1 Ashwin 2083)</t>
+          <t>Asoj 1, 2083 (17 Sep 2026)</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="10" t="inlineStr">
         <is>
-          <t>Nepal Bank Ltd.</t>
+          <t>Nabil Bank Ltd.</t>
         </is>
       </c>
       <c r="B50" s="10" t="inlineStr">
@@ -7395,21 +7301,21 @@
         <v>0.0275</v>
       </c>
       <c r="F50" s="8" t="n">
-        <v>0.03</v>
+        <v>0.028</v>
       </c>
       <c r="G50" s="10" t="inlineStr">
         <is>
-          <t>0.40%</t>
+          <t>Up to 1.375%</t>
         </is>
       </c>
       <c r="H50" s="8" t="n">
-        <v>0.0276</v>
+        <v>0.0285</v>
       </c>
       <c r="I50" s="8" t="n">
-        <v>0.0276</v>
+        <v>0.0285</v>
       </c>
       <c r="J50" s="8" t="n">
-        <v>0.0415</v>
+        <v>0.0455</v>
       </c>
       <c r="K50" s="8" t="n">
         <v>0.0275</v>
@@ -7418,18 +7324,18 @@
         <v>0.0275</v>
       </c>
       <c r="M50" s="8" t="n">
-        <v>0.035</v>
+        <v>0.0301</v>
       </c>
       <c r="N50" s="10" t="inlineStr">
         <is>
-          <t>1st Bhadra 2083</t>
+          <t>17 Aug 2026 (1st Bhadra 2083)</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="10" t="inlineStr">
         <is>
-          <t>Nepal Bank Ltd.</t>
+          <t>Nabil Bank Ltd.</t>
         </is>
       </c>
       <c r="B51" s="10" t="inlineStr">
@@ -7446,44 +7352,44 @@
         <v>3</v>
       </c>
       <c r="E51" s="8" t="n">
-        <v>0.0276</v>
+        <v>0.0275</v>
       </c>
       <c r="F51" s="8" t="n">
+        <v>0.028</v>
+      </c>
+      <c r="G51" s="10" t="inlineStr">
+        <is>
+          <t>Up to 1.375%</t>
+        </is>
+      </c>
+      <c r="H51" s="8" t="n">
+        <v>0.0285</v>
+      </c>
+      <c r="I51" s="8" t="n">
+        <v>0.0285</v>
+      </c>
+      <c r="J51" s="8" t="n">
+        <v>0.0425</v>
+      </c>
+      <c r="K51" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="L51" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="M51" s="8" t="n">
         <v>0.0301</v>
       </c>
-      <c r="G51" s="10" t="inlineStr">
-        <is>
-          <t>0.20%</t>
-        </is>
-      </c>
-      <c r="H51" s="8" t="n">
-        <v>0.0276</v>
-      </c>
-      <c r="I51" s="8" t="n">
-        <v>0.0276</v>
-      </c>
-      <c r="J51" s="8" t="n">
-        <v>0.0415</v>
-      </c>
-      <c r="K51" s="8" t="n">
-        <v>0.0275</v>
-      </c>
-      <c r="L51" s="8" t="n">
-        <v>0.0275</v>
-      </c>
-      <c r="M51" s="8" t="n">
-        <v>0.035</v>
-      </c>
       <c r="N51" s="10" t="inlineStr">
         <is>
-          <t>1st Ashwin 2083</t>
+          <t>17 Sep 2026 (1 Ashwin 2083)</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="10" t="inlineStr">
         <is>
-          <t>Nepal Investment Mega Bank Ltd.</t>
+          <t>Nepal Bank Ltd.</t>
         </is>
       </c>
       <c r="B52" s="10" t="inlineStr">
@@ -7503,26 +7409,24 @@
         <v>0.0275</v>
       </c>
       <c r="F52" s="8" t="n">
-        <v>0.0375</v>
+        <v>0.03</v>
       </c>
       <c r="G52" s="10" t="inlineStr">
         <is>
-          <t>Up to 1.35%</t>
+          <t>0.40%</t>
         </is>
       </c>
       <c r="H52" s="8" t="n">
-        <v>0.029</v>
+        <v>0.0276</v>
       </c>
       <c r="I52" s="8" t="n">
-        <v>0.03</v>
+        <v>0.0276</v>
       </c>
       <c r="J52" s="8" t="n">
-        <v>0.045</v>
-      </c>
-      <c r="K52" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
+        <v>0.0415</v>
+      </c>
+      <c r="K52" s="8" t="n">
+        <v>0.0275</v>
       </c>
       <c r="L52" s="8" t="n">
         <v>0.0275</v>
@@ -7532,14 +7436,14 @@
       </c>
       <c r="N52" s="10" t="inlineStr">
         <is>
-          <t>17 Aug 2026 (1st Bhadra 2083)</t>
+          <t>1st Bhadra 2083</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="10" t="inlineStr">
         <is>
-          <t>Nepal Investment Mega Bank Ltd.</t>
+          <t>Nepal Bank Ltd.</t>
         </is>
       </c>
       <c r="B53" s="10" t="inlineStr">
@@ -7556,29 +7460,27 @@
         <v>3</v>
       </c>
       <c r="E53" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.0276</v>
       </c>
       <c r="F53" s="8" t="n">
-        <v>0.0375</v>
+        <v>0.0301</v>
       </c>
       <c r="G53" s="10" t="inlineStr">
         <is>
-          <t>Up to 1.35%</t>
+          <t>0.20%</t>
         </is>
       </c>
       <c r="H53" s="8" t="n">
-        <v>0.029</v>
+        <v>0.0276</v>
       </c>
       <c r="I53" s="8" t="n">
-        <v>0.03</v>
+        <v>0.0276</v>
       </c>
       <c r="J53" s="8" t="n">
-        <v>0.045</v>
-      </c>
-      <c r="K53" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
+        <v>0.0415</v>
+      </c>
+      <c r="K53" s="8" t="n">
+        <v>0.0275</v>
       </c>
       <c r="L53" s="8" t="n">
         <v>0.0275</v>
@@ -7588,14 +7490,14 @@
       </c>
       <c r="N53" s="10" t="inlineStr">
         <is>
-          <t>17 Sep 2026 (1st Ashwin 2083)</t>
+          <t>1st Ashwin 2083</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="10" t="inlineStr">
         <is>
-          <t>Nepal SBI Bank Ltd.</t>
+          <t>Nepal Investment Mega Bank Ltd.</t>
         </is>
       </c>
       <c r="B54" s="10" t="inlineStr">
@@ -7615,30 +7517,32 @@
         <v>0.0275</v>
       </c>
       <c r="F54" s="8" t="n">
-        <v>0.0279</v>
+        <v>0.0375</v>
       </c>
       <c r="G54" s="10" t="inlineStr">
         <is>
-          <t>Up to 0.75%</t>
+          <t>Up to 1.35%</t>
         </is>
       </c>
       <c r="H54" s="8" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="I54" s="8" t="n">
         <v>0.03</v>
       </c>
-      <c r="I54" s="8" t="n">
-        <v>0.032</v>
-      </c>
       <c r="J54" s="8" t="n">
-        <v>0.04099999999999999</v>
-      </c>
-      <c r="K54" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.045</v>
+      </c>
+      <c r="K54" s="11" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
       </c>
       <c r="L54" s="8" t="n">
         <v>0.0275</v>
       </c>
       <c r="M54" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.035</v>
       </c>
       <c r="N54" s="10" t="inlineStr">
         <is>
@@ -7649,7 +7553,7 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>Nepal SBI Bank Ltd.</t>
+          <t>Nepal Investment Mega Bank Ltd.</t>
         </is>
       </c>
       <c r="B55" s="10" t="inlineStr">
@@ -7669,30 +7573,32 @@
         <v>0.0275</v>
       </c>
       <c r="F55" s="8" t="n">
-        <v>0.0279</v>
+        <v>0.0375</v>
       </c>
       <c r="G55" s="10" t="inlineStr">
         <is>
-          <t>Up to 0.75%</t>
+          <t>Up to 1.35%</t>
         </is>
       </c>
       <c r="H55" s="8" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="I55" s="8" t="n">
         <v>0.03</v>
       </c>
-      <c r="I55" s="8" t="n">
-        <v>0.032</v>
-      </c>
       <c r="J55" s="8" t="n">
-        <v>0.04099999999999999</v>
-      </c>
-      <c r="K55" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.045</v>
+      </c>
+      <c r="K55" s="11" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
       </c>
       <c r="L55" s="8" t="n">
         <v>0.0275</v>
       </c>
       <c r="M55" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.035</v>
       </c>
       <c r="N55" s="10" t="inlineStr">
         <is>
@@ -7703,7 +7609,7 @@
     <row r="56">
       <c r="A56" s="10" t="inlineStr">
         <is>
-          <t>Prabhu Bank Ltd.</t>
+          <t>Nepal SBI Bank Ltd.</t>
         </is>
       </c>
       <c r="B56" s="10" t="inlineStr">
@@ -7723,21 +7629,21 @@
         <v>0.0275</v>
       </c>
       <c r="F56" s="8" t="n">
+        <v>0.0279</v>
+      </c>
+      <c r="G56" s="10" t="inlineStr">
+        <is>
+          <t>Up to 0.75%</t>
+        </is>
+      </c>
+      <c r="H56" s="8" t="n">
         <v>0.03</v>
       </c>
-      <c r="G56" s="10" t="inlineStr">
-        <is>
-          <t>Up to 0.10%</t>
-        </is>
-      </c>
-      <c r="H56" s="8" t="n">
-        <v>0.0275</v>
-      </c>
       <c r="I56" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.032</v>
       </c>
       <c r="J56" s="8" t="n">
-        <v>0.0455</v>
+        <v>0.04099999999999999</v>
       </c>
       <c r="K56" s="8" t="n">
         <v>0.0275</v>
@@ -7750,14 +7656,14 @@
       </c>
       <c r="N56" s="10" t="inlineStr">
         <is>
-          <t>17 Aug 2026 (01 Bhadra 2083)</t>
+          <t>17 Aug 2026 (1st Bhadra 2083)</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="10" t="inlineStr">
         <is>
-          <t>Prabhu Bank Ltd.</t>
+          <t>Nepal SBI Bank Ltd.</t>
         </is>
       </c>
       <c r="B57" s="10" t="inlineStr">
@@ -7777,21 +7683,21 @@
         <v>0.0275</v>
       </c>
       <c r="F57" s="8" t="n">
+        <v>0.0279</v>
+      </c>
+      <c r="G57" s="10" t="inlineStr">
+        <is>
+          <t>Up to 0.75%</t>
+        </is>
+      </c>
+      <c r="H57" s="8" t="n">
         <v>0.03</v>
       </c>
-      <c r="G57" s="10" t="inlineStr">
-        <is>
-          <t>Up to 0.10%</t>
-        </is>
-      </c>
-      <c r="H57" s="8" t="n">
-        <v>0.0275</v>
-      </c>
       <c r="I57" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.032</v>
       </c>
       <c r="J57" s="8" t="n">
-        <v>0.0455</v>
+        <v>0.04099999999999999</v>
       </c>
       <c r="K57" s="8" t="n">
         <v>0.0275</v>
@@ -7804,14 +7710,14 @@
       </c>
       <c r="N57" s="10" t="inlineStr">
         <is>
-          <t>17 Sep 2026 (01 Ashwin 2083)</t>
+          <t>17 Sep 2026 (1st Ashwin 2083)</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="10" t="inlineStr">
         <is>
-          <t>Prime Commercial Bank Ltd.</t>
+          <t>Prabhu Bank Ltd.</t>
         </is>
       </c>
       <c r="B58" s="10" t="inlineStr">
@@ -7828,24 +7734,24 @@
         <v>2</v>
       </c>
       <c r="E58" s="8" t="n">
-        <v>0.0276</v>
+        <v>0.0275</v>
       </c>
       <c r="F58" s="8" t="n">
-        <v>0.0302</v>
+        <v>0.03</v>
       </c>
       <c r="G58" s="10" t="inlineStr">
         <is>
-          <t>Up to 1.37%</t>
+          <t>Up to 0.10%</t>
         </is>
       </c>
       <c r="H58" s="8" t="n">
-        <v>0.029</v>
+        <v>0.0275</v>
       </c>
       <c r="I58" s="8" t="n">
-        <v>0.03</v>
+        <v>0.0275</v>
       </c>
       <c r="J58" s="8" t="n">
-        <v>0.04</v>
+        <v>0.0455</v>
       </c>
       <c r="K58" s="8" t="n">
         <v>0.0275</v>
@@ -7858,14 +7764,14 @@
       </c>
       <c r="N58" s="10" t="inlineStr">
         <is>
-          <t>01st Bhadra 2083 (17 Aug 2026)</t>
+          <t>17 Aug 2026 (01 Bhadra 2083)</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="10" t="inlineStr">
         <is>
-          <t>Prime Commercial Bank Ltd.</t>
+          <t>Prabhu Bank Ltd.</t>
         </is>
       </c>
       <c r="B59" s="10" t="inlineStr">
@@ -7882,24 +7788,24 @@
         <v>3</v>
       </c>
       <c r="E59" s="8" t="n">
-        <v>0.0276</v>
+        <v>0.0275</v>
       </c>
       <c r="F59" s="8" t="n">
-        <v>0.0302</v>
+        <v>0.03</v>
       </c>
       <c r="G59" s="10" t="inlineStr">
         <is>
-          <t>Up to 1.37%</t>
+          <t>Up to 0.10%</t>
         </is>
       </c>
       <c r="H59" s="8" t="n">
-        <v>0.029</v>
+        <v>0.0275</v>
       </c>
       <c r="I59" s="8" t="n">
-        <v>0.03</v>
+        <v>0.0275</v>
       </c>
       <c r="J59" s="8" t="n">
-        <v>0.04</v>
+        <v>0.0455</v>
       </c>
       <c r="K59" s="8" t="n">
         <v>0.0275</v>
@@ -7912,14 +7818,14 @@
       </c>
       <c r="N59" s="10" t="inlineStr">
         <is>
-          <t>01st Ashwin 2083 (17 Sep 2026)</t>
+          <t>17 Sep 2026 (01 Ashwin 2083)</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="10" t="inlineStr">
         <is>
-          <t>Rastriya Banijya Bank Ltd.</t>
+          <t>Prime Commercial Bank Ltd.</t>
         </is>
       </c>
       <c r="B60" s="10" t="inlineStr">
@@ -7936,21 +7842,21 @@
         <v>2</v>
       </c>
       <c r="E60" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.0276</v>
       </c>
       <c r="F60" s="8" t="n">
-        <v>0.028</v>
+        <v>0.0302</v>
       </c>
       <c r="G60" s="10" t="inlineStr">
         <is>
-          <t>0.50%</t>
+          <t>Up to 1.37%</t>
         </is>
       </c>
       <c r="H60" s="8" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="I60" s="8" t="n">
         <v>0.03</v>
-      </c>
-      <c r="I60" s="8" t="n">
-        <v>0.0315</v>
       </c>
       <c r="J60" s="8" t="n">
         <v>0.04</v>
@@ -7962,18 +7868,18 @@
         <v>0.0275</v>
       </c>
       <c r="M60" s="8" t="n">
-        <v>0.03</v>
+        <v>0.0275</v>
       </c>
       <c r="N60" s="10" t="inlineStr">
         <is>
-          <t>2083 Bhadra 01 (17 Aug 2026)</t>
+          <t>01st Bhadra 2083 (17 Aug 2026)</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="10" t="inlineStr">
         <is>
-          <t>Rastriya Banijya Bank Ltd.</t>
+          <t>Prime Commercial Bank Ltd.</t>
         </is>
       </c>
       <c r="B61" s="10" t="inlineStr">
@@ -7990,21 +7896,21 @@
         <v>3</v>
       </c>
       <c r="E61" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.0276</v>
       </c>
       <c r="F61" s="8" t="n">
-        <v>0.028</v>
+        <v>0.0302</v>
       </c>
       <c r="G61" s="10" t="inlineStr">
         <is>
-          <t>0.50%</t>
+          <t>Up to 1.37%</t>
         </is>
       </c>
       <c r="H61" s="8" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="I61" s="8" t="n">
         <v>0.03</v>
-      </c>
-      <c r="I61" s="8" t="n">
-        <v>0.0315</v>
       </c>
       <c r="J61" s="8" t="n">
         <v>0.04</v>
@@ -8016,18 +7922,18 @@
         <v>0.0275</v>
       </c>
       <c r="M61" s="8" t="n">
-        <v>0.03</v>
+        <v>0.0275</v>
       </c>
       <c r="N61" s="10" t="inlineStr">
         <is>
-          <t>2083 Asoj 01 (17 Sep 2026)</t>
+          <t>01st Ashwin 2083 (17 Sep 2026)</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="10" t="inlineStr">
         <is>
-          <t>Sanima Bank Ltd.</t>
+          <t>Rastriya Banijya Bank Ltd.</t>
         </is>
       </c>
       <c r="B62" s="10" t="inlineStr">
@@ -8051,17 +7957,17 @@
       </c>
       <c r="G62" s="10" t="inlineStr">
         <is>
-          <t>Up to 1.375%</t>
+          <t>0.50%</t>
         </is>
       </c>
       <c r="H62" s="8" t="n">
-        <v>0.028</v>
+        <v>0.03</v>
       </c>
       <c r="I62" s="8" t="n">
-        <v>0.028</v>
+        <v>0.0315</v>
       </c>
       <c r="J62" s="8" t="n">
-        <v>0.045</v>
+        <v>0.04</v>
       </c>
       <c r="K62" s="8" t="n">
         <v>0.0275</v>
@@ -8070,18 +7976,18 @@
         <v>0.0275</v>
       </c>
       <c r="M62" s="8" t="n">
-        <v>0.033</v>
+        <v>0.03</v>
       </c>
       <c r="N62" s="10" t="inlineStr">
         <is>
-          <t>Bhadra 2083</t>
+          <t>2083 Bhadra 01 (17 Aug 2026)</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="10" t="inlineStr">
         <is>
-          <t>Sanima Bank Ltd.</t>
+          <t>Rastriya Banijya Bank Ltd.</t>
         </is>
       </c>
       <c r="B63" s="10" t="inlineStr">
@@ -8105,17 +8011,17 @@
       </c>
       <c r="G63" s="10" t="inlineStr">
         <is>
-          <t>Up to 1.375%</t>
+          <t>0.50%</t>
         </is>
       </c>
       <c r="H63" s="8" t="n">
-        <v>0.028</v>
+        <v>0.03</v>
       </c>
       <c r="I63" s="8" t="n">
-        <v>0.028</v>
+        <v>0.0315</v>
       </c>
       <c r="J63" s="8" t="n">
-        <v>0.045</v>
+        <v>0.04</v>
       </c>
       <c r="K63" s="8" t="n">
         <v>0.0275</v>
@@ -8124,18 +8030,18 @@
         <v>0.0275</v>
       </c>
       <c r="M63" s="8" t="n">
-        <v>0.0351</v>
+        <v>0.03</v>
       </c>
       <c r="N63" s="10" t="inlineStr">
         <is>
-          <t>Ashwin 1, 2083</t>
+          <t>2083 Asoj 01 (17 Sep 2026)</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="10" t="inlineStr">
         <is>
-          <t>Siddhartha Bank Ltd.</t>
+          <t>Sanima Bank Ltd.</t>
         </is>
       </c>
       <c r="B64" s="10" t="inlineStr">
@@ -8155,43 +8061,41 @@
         <v>0.0275</v>
       </c>
       <c r="F64" s="8" t="n">
-        <v>0.0305</v>
+        <v>0.028</v>
       </c>
       <c r="G64" s="10" t="inlineStr">
         <is>
-          <t>Up to 0.25%</t>
+          <t>Up to 1.375%</t>
         </is>
       </c>
       <c r="H64" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.028</v>
       </c>
       <c r="I64" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.028</v>
       </c>
       <c r="J64" s="8" t="n">
-        <v>0.03759999999999999</v>
-      </c>
-      <c r="K64" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
+        <v>0.045</v>
+      </c>
+      <c r="K64" s="8" t="n">
+        <v>0.0275</v>
       </c>
       <c r="L64" s="8" t="n">
         <v>0.0275</v>
       </c>
       <c r="M64" s="8" t="n">
-        <v>0.0305</v>
+        <v>0.033</v>
       </c>
       <c r="N64" s="10" t="inlineStr">
         <is>
-          <t>17 Aug 2026</t>
+          <t>Bhadra 2083</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="10" t="inlineStr">
         <is>
-          <t>Siddhartha Bank Ltd.</t>
+          <t>Sanima Bank Ltd.</t>
         </is>
       </c>
       <c r="B65" s="10" t="inlineStr">
@@ -8211,43 +8115,41 @@
         <v>0.0275</v>
       </c>
       <c r="F65" s="8" t="n">
-        <v>0.0305</v>
+        <v>0.028</v>
       </c>
       <c r="G65" s="10" t="inlineStr">
         <is>
-          <t>Up to 0.25%</t>
+          <t>Up to 1.375%</t>
         </is>
       </c>
       <c r="H65" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.028</v>
       </c>
       <c r="I65" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.028</v>
       </c>
       <c r="J65" s="8" t="n">
-        <v>0.03759999999999999</v>
-      </c>
-      <c r="K65" s="11" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
+        <v>0.045</v>
+      </c>
+      <c r="K65" s="8" t="n">
+        <v>0.0275</v>
       </c>
       <c r="L65" s="8" t="n">
         <v>0.0275</v>
       </c>
       <c r="M65" s="8" t="n">
-        <v>0.0305</v>
+        <v>0.0351</v>
       </c>
       <c r="N65" s="10" t="inlineStr">
         <is>
-          <t>17 Sep 2026</t>
+          <t>Ashwin 1, 2083</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="10" t="inlineStr">
         <is>
-          <t>Standard Chartered Bank Nepal Ltd.</t>
+          <t>Siddhartha Bank Ltd.</t>
         </is>
       </c>
       <c r="B66" s="10" t="inlineStr">
@@ -8267,7 +8169,7 @@
         <v>0.0275</v>
       </c>
       <c r="F66" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.0305</v>
       </c>
       <c r="G66" s="10" t="inlineStr">
         <is>
@@ -8281,7 +8183,7 @@
         <v>0.0275</v>
       </c>
       <c r="J66" s="8" t="n">
-        <v>0.038</v>
+        <v>0.03759999999999999</v>
       </c>
       <c r="K66" s="11" t="inlineStr">
         <is>
@@ -8292,7 +8194,7 @@
         <v>0.0275</v>
       </c>
       <c r="M66" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.0305</v>
       </c>
       <c r="N66" s="10" t="inlineStr">
         <is>
@@ -8303,7 +8205,7 @@
     <row r="67">
       <c r="A67" s="10" t="inlineStr">
         <is>
-          <t>Standard Chartered Bank Nepal Ltd.</t>
+          <t>Siddhartha Bank Ltd.</t>
         </is>
       </c>
       <c r="B67" s="10" t="inlineStr">
@@ -8323,41 +8225,153 @@
         <v>0.0275</v>
       </c>
       <c r="F67" s="8" t="n">
-        <v>0.0275</v>
+        <v>0.0305</v>
       </c>
       <c r="G67" s="10" t="inlineStr">
         <is>
+          <t>Up to 0.25%</t>
+        </is>
+      </c>
+      <c r="H67" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="I67" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="J67" s="8" t="n">
+        <v>0.03759999999999999</v>
+      </c>
+      <c r="K67" s="11" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="L67" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="M67" s="8" t="n">
+        <v>0.0305</v>
+      </c>
+      <c r="N67" s="10" t="inlineStr">
+        <is>
+          <t>17 Sep 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="10" t="inlineStr">
+        <is>
+          <t>Standard Chartered Bank Nepal Ltd.</t>
+        </is>
+      </c>
+      <c r="B68" s="10" t="inlineStr">
+        <is>
+          <t>Commercial Banks</t>
+        </is>
+      </c>
+      <c r="C68" s="10" t="inlineStr">
+        <is>
+          <t>Bhadra 2083</t>
+        </is>
+      </c>
+      <c r="D68" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E68" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="F68" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="G68" s="10" t="inlineStr">
+        <is>
+          <t>Up to 0.25%</t>
+        </is>
+      </c>
+      <c r="H68" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="I68" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="J68" s="8" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="K68" s="11" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="L68" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="M68" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="N68" s="10" t="inlineStr">
+        <is>
+          <t>17 Aug 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="10" t="inlineStr">
+        <is>
+          <t>Standard Chartered Bank Nepal Ltd.</t>
+        </is>
+      </c>
+      <c r="B69" s="10" t="inlineStr">
+        <is>
+          <t>Commercial Banks</t>
+        </is>
+      </c>
+      <c r="C69" s="10" t="inlineStr">
+        <is>
+          <t>Ashwin 2083</t>
+        </is>
+      </c>
+      <c r="D69" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E69" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="F69" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="G69" s="10" t="inlineStr">
+        <is>
           <t>Up to 0.20%</t>
         </is>
       </c>
-      <c r="H67" s="8" t="n">
-        <v>0.0275</v>
-      </c>
-      <c r="I67" s="8" t="n">
-        <v>0.0275</v>
-      </c>
-      <c r="J67" s="8" t="n">
+      <c r="H69" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="I69" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="J69" s="8" t="n">
         <v>0.0375</v>
       </c>
-      <c r="K67" s="11" t="inlineStr">
+      <c r="K69" s="11" t="inlineStr">
         <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="L67" s="8" t="n">
-        <v>0.0275</v>
-      </c>
-      <c r="M67" s="8" t="n">
-        <v>0.0275</v>
-      </c>
-      <c r="N67" s="10" t="inlineStr">
+      <c r="L69" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="M69" s="8" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="N69" s="10" t="inlineStr">
         <is>
           <t>17 Sep 2026</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N67"/>
+  <autoFilter ref="A1:N69"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>